<commit_message>
feat(ml): export RainNext24h labels to Gold ML
- export_rain_labels: read Silver Open-Meteo hourly data for the 8 canonical
  locations (refuse to publish on any missing location-month), build labels
  with rain_labels (1 mm over (t, t+24h], 24 valid hours, UTC splits with
  boundary purge), and write gold/ml_labels/rain_next24h_labels_v1.parquet
  plus a JSON manifest with scope, counts, and positive rates.
- tests: exact Yes/No origins around a rain hour, boundary purge counts, and
  refusal on an incomplete Silver snapshot.
- docs: naming conventions, rain label, progress; workbook ID 22.

Tests: make test 70 passed.
Real data 2016-2025: 700,800 usable labels (train 560,832 / validation
70,080 / test 69,888; positive 50.9% / 49.4% / 49.0%), 576 purged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Phan_cong_cong_viec_DW_khi_tuong.xlsx
+++ b/Phan_cong_cong_viec_DW_khi_tuong.xlsx
@@ -3031,11 +3031,11 @@
         </is>
       </c>
       <c r="N26" s="23" t="n">
-        <v>40</v>
+        <v>95</v>
       </c>
       <c r="O26" s="24" t="inlineStr">
         <is>
-          <t>21/10: scripts/rain_labels.py (cửa sổ (t,t+24h], ngưỡng 1 mm, thiếu giờ thì không nhãn, loại mẫu ở ranh giới tập) + 10 unit test. Chạy thử trên Open-Meteo 2016–2025: 700.800 nhãn dùng được, 576 bị loại ở ranh giới. Chưa xuất bảng nhãn từ Silver/Gold</t>
+          <t>21/10: gold/ml_labels/rain_next24h_labels_v1.parquet + manifest: 700.800 nhãn dùng được (train 560.832 / val 70.080 / test 69.888; Yes 50,9% / 49,4% / 49,0%), 576 mẫu loại ở ranh giới. Test t/t+1/t+24/t+25, thiếu giờ, ranh giới. Do N1/N2 làm thay N3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(ml): add RainNext24h EDA notebook and notebook environment
- rain_eda: join labels with Silver Open-Meteo variables at origin t and
  trailing derivations (past-24 h rain, 24 h pressure change, dew-point
  depression) per location on a gap-checked grid; class balance, month x
  location rates, missingness, target distribution, standardized mean
  differences, and binned rates (train split by default).
- tests: past/present-only inputs (changing data after t leaves t unchanged),
  gap handling, split filtering, duplicate rejection.
- notebooks/eda_rain_next24h.ipynb: executed on the real Silver/Gold data;
  charts use the validated reference palette and each has a table.
- requirements-notebook.in/.txt (uv 0.8.22, hashed), make notebook-setup /
  notebook-run, .venv-*/ ignored, development docs; workbook ID 21.

Tests: make test 74 passed; notebook executed with 0 errors.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Phan_cong_cong_viec_DW_khi_tuong.xlsx
+++ b/Phan_cong_cong_viec_DW_khi_tuong.xlsx
@@ -2979,13 +2979,19 @@
         <f aca="false">'Tổng quan'!$E$11+(C25-1)*7+4</f>
         <v>46339</v>
       </c>
-      <c r="M25" s="22" t="s">
-        <v>62</v>
+      <c r="M25" s="22" t="inlineStr">
+        <is>
+          <t>Đang làm</t>
+        </is>
       </c>
       <c r="N25" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O25" s="24"/>
+        <v>90</v>
+      </c>
+      <c r="O25" s="24" t="inlineStr">
+        <is>
+          <t>21/10: notebooks/eda_rain_next24h.ipynb (chạy trên dữ liệu thật, chỉ dùng tập train để chọn biến): mùa vụ mạnh (T8 78%, T12 26%), giờ trong ngày gần như không ảnh hưởng, biến tách tốt nhất: điểm sương, mưa 24h trước, độ ẩm, áp suất. Logic trong scripts/rain_eda.py có test. Do N1/N2 làm thay N3</t>
+        </is>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="19" t="n">

</xml_diff>

<commit_message>
feat(ml): build leakage-free RainNext24h feature dataset (ID 23)
- scripts/build_rain_features.py: 22 Open-Meteo features per location on a
  gap-checked hourly grid (values at t, 3h/6h lags, 3/6/12/24h trailing
  rain, 6h means, 3h/24h pressure change, UTC+7 hour/month). Writes
  gold/ml_features/cart_rain_{train_2016_2023,val_2024,test_2025}_v1.parquet
  plus a manifest with ordered features and units.
- tests/test_rain_features.py: post-t changes leave features unchanged,
  gaps give NaN, no cross-location lags, local calendar, export.
- Real 2016-2025 run: 700,800 rows = usable labels; missing values only
  in the first 24 origin hours of 2016.
- Docs: feature v1 section in rain-label.md, naming fix for ml_features,
  README/architecture status refresh, progress entries, workbook ID 23.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Phan_cong_cong_viec_DW_khi_tuong.xlsx
+++ b/Phan_cong_cong_viec_DW_khi_tuong.xlsx
@@ -3083,13 +3083,19 @@
         <f aca="false">'Tổng quan'!$E$11+(C27-1)*7+4</f>
         <v>46339</v>
       </c>
-      <c r="M27" s="22" t="s">
-        <v>62</v>
+      <c r="M27" s="22" t="inlineStr">
+        <is>
+          <t>Đang làm</t>
+        </is>
       </c>
       <c r="N27" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O27" s="24"/>
+        <v>90</v>
+      </c>
+      <c r="O27" s="24" t="inlineStr">
+        <is>
+          <t>21/10: gold/ml_features/cart_rain_{train_2016_2023,val_2024,test_2025}_v1.parquet + manifest: 22 đặc trưng chỉ từ Open-Meteo (giá trị tại t, trễ 3/6h, mưa 3/6/12/24h trước, TB 6h, biến thiên áp suất 3h/24h, giờ/tháng địa phương). 700.800 dòng = đúng số nhãn dùng được; thiếu giá trị chỉ ở 24 giờ đầu 2016 (192 dòng). Test chống rò rỉ, thiếu giờ, không lẫn vị trí. Do N1/N2 làm thay N3</t>
+        </is>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="19" t="n">

</xml_diff>

<commit_message>
feat(ml): train and tune CART RainNext24h on train/validation (ID 28)
- scripts/train_cart.py: one-hot location + 22 features -> DecisionTree;
  120-config grid fit on train 2016-2023, selected by validation 2024 F1
  (ties within 0.005 -> shallowest tree), probability threshold chosen
  on validation, baselines, model.joblib + report.json in gold/ml_models.
  The test split is refused.
- tests/test_train_cart.py: metrics edge cases, tie rules, test split
  never read, reproducible training and model reload.
- Real run: max_depth=8, min_samples_leaf=50, class_weight=balanced,
  ccp_alpha=1e-4, 88 leaves, threshold 0.40; validation F1 0.786,
  recall 0.822 (persistence baseline F1 0.753).
- Docs: rain-label.md CART v1 section, naming row, README/architecture,
  progress entry, workbook ID 28.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Phan_cong_cong_viec_DW_khi_tuong.xlsx
+++ b/Phan_cong_cong_viec_DW_khi_tuong.xlsx
@@ -3321,13 +3321,19 @@
         <f aca="false">'Tổng quan'!$E$11+(C32-1)*7+4</f>
         <v>46353</v>
       </c>
-      <c r="M32" s="22" t="s">
-        <v>62</v>
+      <c r="M32" s="22" t="inlineStr">
+        <is>
+          <t>Đang làm</t>
+        </is>
       </c>
       <c r="N32" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O32" s="24"/>
+        <v>90</v>
+      </c>
+      <c r="O32" s="24" t="inlineStr">
+        <is>
+          <t>21/10: gold/ml_models/cart_rain_next24h_v1 (model.joblib + report.json). Lưới 120 cấu hình fit trên train 2016-2023, chọn trên validation 2024 theo F1: max_depth=8, min_samples_leaf=50, class_weight=balanced, ccp_alpha=1e-4, 88 lá, ngưỡng xác suất 0,40. Validation: Precision 0,752 / Recall 0,822 / F1 0,786 (mốc dự báo theo hiện trạng F1 0,753). Chưa đọc tập test. Do N1/N2 làm thay N3</t>
+        </is>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="19" t="n">

</xml_diff>

<commit_message>
feat(ml): evaluate frozen CART once on test 2025 (ID 29)
- scripts/evaluate_cart_test.py: loads the ID 28 model and threshold,
  checks the feature list and that the model reproduces its validation
  confusion matrix before reading test, refuses a second evaluation, and
  writes test_evaluation.json + test_predictions.parquet.
- tests/test_evaluate_cart_test.py: frozen threshold, single run,
  swapped model rejected before test is read, feature mismatch rejected.
- Real run (69,888 test rows): precision 0.756, recall 0.795, F1 0.775
  at threshold 0.40; persistence baseline F1 0.726; dry season F1 0.621.
- Docs: rain-label.md test section, naming row, README/architecture,
  progress entry, workbook ID 29.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Phan_cong_cong_viec_DW_khi_tuong.xlsx
+++ b/Phan_cong_cong_viec_DW_khi_tuong.xlsx
@@ -3373,13 +3373,19 @@
         <f aca="false">'Tổng quan'!$E$11+(C33-1)*7+4</f>
         <v>46353</v>
       </c>
-      <c r="M33" s="22" t="s">
-        <v>62</v>
+      <c r="M33" s="22" t="inlineStr">
+        <is>
+          <t>Đang làm</t>
+        </is>
       </c>
       <c r="N33" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O33" s="24"/>
+        <v>90</v>
+      </c>
+      <c r="O33" s="24" t="inlineStr">
+        <is>
+          <t>21/10: đánh giá 1 lần trên test 2025 với model + ngưỡng 0,40 đã chốt từ validation (không chỉnh ngưỡng bằng test). 69.888/69.888 mẫu. TP 27.254 / FP 8.782 / TN 26.840 / FN 7.012; Accuracy 0,774, Precision 0,756, Recall 0,795, F1 0,775 (dự báo theo hiện trạng F1 0,726). Mùa mưa F1 0,835, mùa khô 0,621. gold/ml_models/cart_rain_next24h_v1/test_evaluation.json. Do N1/N2 làm thay N3</t>
+        </is>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="19" t="n">

</xml_diff>

<commit_message>
feat(ml): CART v1 tree figure, rules, and missed-rain profile (ID 30)
- scripts/cart_rules.py: rules from the evaluated artifact with merged
  per-variable intervals in real units, location wording for one-hot
  splits, node table, decision paths, rain-onset hours, and a missed-rain
  profile.
- notebooks/cart_tree_rules.ipynb (executed): SHA-256 check against the
  ID 29 evaluation, first 3 tree levels, 88 rules, importances, four
  test-2025 examples, and an error profile on validation 2024.
- Correction: the first interpretation generalized "rain without warning"
  from one extreme example; validation shows most misses are light rain
  near the threshold, and wind direction was never assessed in the EDA.
- Makefile notebook-run accepts NOTEBOOK=...; docs, progress, workbook ID 30.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Phan_cong_cong_viec_DW_khi_tuong.xlsx
+++ b/Phan_cong_cong_viec_DW_khi_tuong.xlsx
@@ -3425,13 +3425,19 @@
         <f aca="false">'Tổng quan'!$E$11+(C34-1)*7+4</f>
         <v>46353</v>
       </c>
-      <c r="M34" s="22" t="s">
-        <v>62</v>
+      <c r="M34" s="22" t="inlineStr">
+        <is>
+          <t>Đang làm</t>
+        </is>
       </c>
       <c r="N34" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O34" s="24"/>
+        <v>90</v>
+      </c>
+      <c r="O34" s="24" t="inlineStr">
+        <is>
+          <t>21/10: notebooks/cart_tree_rules.ipynb (kiểm tra SHA-256 đúng model đã đánh giá ở ID 29): hình 3 tầng đầu cây, 88 luật bằng tên + đơn vị thật, độ quan trọng, 4 ví dụ test 2025 (TP/FP/FN cực đoan/FN điển hình), hồ sơ ca bỏ sót trên validation 2024: 64% dưới 5 mm, 55% xác suất 0,30-0,40, mưa sau 24h khô chỉ bắt được 17% (mùa khô 2,6%). Đã sửa lời diễn giải «mưa không báo trước» (suy từ 1 ví dụ). Do N1/N2 làm thay N3</t>
+        </is>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="19" t="n">

</xml_diff>

<commit_message>
feat(dw): load CART predictions with dim_model and prediction-vs-actual view (ID 31)
- sql/04_predictions.sql (idempotent): dim_model; fact_weather_prediction
  gains model_key, UTC origin, target window, horizon, threshold, split,
  unique (model, location, origin) and CHECKs; observation index for
  24 h window sums; vw_prediction_vs_actual (NULL when incomplete).
- scripts/load_predictions.py: upserts dim_model, validates inputs,
  Vietnam-local keys, replaces the (model, split) scope in one transaction.
- tests: 7 unit + 3 integration (rerun, retraction, window boundaries,
  constraints).
- Real DW: 69,888 test 2025 predictions, rerun duplicate-free.
- The view's independent reconciliation exposed a label bug in ID 22:
  float sums turn exactly-1.0 mm windows into No (5,147 labels, 0.73%).
  Recorded in progress.md; fix follows.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Phan_cong_cong_viec_DW_khi_tuong.xlsx
+++ b/Phan_cong_cong_viec_DW_khi_tuong.xlsx
@@ -3479,13 +3479,19 @@
         <f aca="false">'Tổng quan'!$E$11+(C35-1)*7+4</f>
         <v>46360</v>
       </c>
-      <c r="M35" s="22" t="s">
-        <v>62</v>
+      <c r="M35" s="22" t="inlineStr">
+        <is>
+          <t>Đang làm</t>
+        </is>
       </c>
       <c r="N35" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O35" s="24"/>
+        <v>90</v>
+      </c>
+      <c r="O35" s="24" t="inlineStr">
+        <is>
+          <t>22/10: sql/04_predictions.sql (dim_model, khóa duy nhất model × vị trí × origin UTC, cửa sổ mục tiêu, view vw_prediction_vs_actual) + scripts/load_predictions.py. Đã nạp 69.888 dự đoán test 2025, chạy lại không trùng. View đối chiếu phát hiện lỗi nhãn ID 22 (tổng đúng 1,0 mm bị gán Không mưa, 0,73% nhãn); đang sửa. Do N1/N2 làm thay N3</t>
+        </is>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="19" t="n">

</xml_diff>

<commit_message>
docs: record boundary, Recall, and ERA5 decisions after the audit
- Pre-merger boundaries were already decided by the N2 owner of IDs 4/11;
  remove the "pending team confirmation" wording added by the audit.
- Recall operating point: highest validation precision with validation
  recall >= 0.85 (0.36 for CART v1); 0.40 stays the official test result.
- ERA5 request scope accepted; download waits for N3's CDS account.
- Add the N3 review checklist to rain-label.md; workbook notes updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Phan_cong_cong_viec_DW_khi_tuong.xlsx
+++ b/Phan_cong_cong_viec_DW_khi_tuong.xlsx
@@ -2131,7 +2131,7 @@
       </c>
       <c r="O8" s="24" t="inlineStr">
         <is>
-          <t>22/10: chưa bắt đầu, trễ hạn tuần 1. 21/10 N1/N2 đề xuất đổi phạm vi sang ranh giới trước sáp nhập (63 tỉnh) vì giai đoạn nghiên cứu gần như toàn bộ trước 1/7/2025; chờ nhóm xác nhận. Nguồn ứng viên và tiêu chí: task-specs §7; kế hoạch: business-requirements §5a</t>
+          <t>22/10: chưa bắt đầu, trễ hạn tuần 1. Phạm vi đã chốt 21/10 (N2): dùng ranh giới trước sáp nhập (63 tỉnh), không làm ranh giới sau 1/7/2025, vì giai đoạn nghiên cứu gần như toàn bộ trước sáp nhập. Nguồn ứng viên và tiêu chí: docs/task-specs-weeks-2-5.md §7</t>
         </is>
       </c>
     </row>
@@ -2181,7 +2181,7 @@
       </c>
       <c r="O9" s="24" t="inlineStr">
         <is>
-          <t>22/10: chưa bắt đầu, trễ hạn tuần 1; thiếu ERA5 nên chưa đạt mục tiêu đa định dạng (NetCDF). Đề xuất phạm vi và thứ tự (ID 4 → ID 5 → ID 14/15) ở business-requirements §5a; chỉ tải khi N3 xác nhận phạm vi</t>
+          <t>22/10: chưa bắt đầu, trễ hạn tuần 1. Phạm vi đã thống nhất 22/10 (N1/N2, chờ N3 xác nhận): ERA5 hourly single levels, vùng 19,5–23,5°N, 102,5–107,5°E, biến t2m, d2m, tp, sp, u10, v10, tcc, 2016–2025, NetCDF. Việc cần N3: tạo tài khoản Copernicus CDS và chấp nhận giấy phép; chưa tải khi chưa có tài khoản</t>
         </is>
       </c>
     </row>
@@ -2493,7 +2493,7 @@
       </c>
       <c r="O15" s="24" t="inlineStr">
         <is>
-          <t>21/10: mã/tọa độ trạm đã xác minh (Meteostat + NOAA ISD). Hợp lệ: HAN 48820, HPH 48826, TNG 48831, LCA 48803; dim_station 12 trạm (thêm 48823 Nam Định cho mưa ngày). 22/10: 48820 = sân bay Nội Bài (22,0 km, vai trò nearest_available); thêm station_role, distance_km (sql/05). Khoảng cách tính bằng haversine, không dùng GeoPandas. Tỉnh cũ-mới: không làm theo đề xuất ranh giới trước sáp nhập, chờ nhóm xác nhận</t>
+          <t>21/10: mã/tọa độ trạm đã xác minh (Meteostat + NOAA ISD). Hợp lệ: HAN 48820, HPH 48826, TNG 48831, LCA 48803; dim_station 12 trạm (thêm 48823 Nam Định cho mưa ngày). 22/10: 48820 = sân bay Nội Bài (22,0 km, vai trò nearest_available); thêm station_role, distance_km (sql/05). Khoảng cách tính bằng haversine, không dùng GeoPandas. Tỉnh: đã chốt 21/10 chỉ dùng tỉnh trước sáp nhập, không làm ánh xạ tỉnh cũ-mới</t>
         </is>
       </c>
     </row>
@@ -4237,7 +4237,7 @@
       </c>
       <c r="F9" s="24" t="inlineStr">
         <is>
-          <t>21/10: N1/N2 đề xuất dùng ranh giới trước sáp nhập (63 tỉnh); DimLocation chỉ lưu tỉnh cũ. Chờ nhóm xác nhận</t>
+          <t>21/10: đã chốt (N2) dùng ranh giới trước sáp nhập (63 tỉnh); DimLocation chỉ lưu tỉnh cũ, không lưu tỉnh mới</t>
         </is>
       </c>
     </row>
@@ -4299,7 +4299,7 @@
       </c>
       <c r="F12" s="24" t="inlineStr">
         <is>
-          <t>21/10: ngưỡng 0,40 chọn trên 2024 theo F1 (Recall 0,82); chưa có mục tiêu Recall định lượng (đề xuất chờ duyệt)</t>
+          <t>22/10: ngưỡng 0,40 chọn trên 2024 theo F1 (Recall 0,82) là kết quả test chính thức. Thêm điểm vận hành ưu tiên Recall: Recall validation ≥ 0,85 và Precision cao nhất → 0,36 (Recall 0,88). Do N1/N2 chốt thay N3, chờ N3 duyệt</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(spatial): pre-merger province boundaries to Bronze and Silver (ID 4)
- scripts/ingest_boundaries.py: geoBoundaries VNM ADM1 pinned to commit
  9469f09 (2008, 64 units = 63 provinces + Côn Đảo), received bytes in
  Bronze with a manifest (SHA-256, license note, CRS); Silver subset of the
  25 northern provinces (Decisions 368/369/QĐ-TTg) with the 8 research
  provinces flagged. Validates CRS, unit count, names, geometry, and that
  each research point lies in its dim_location.province before publishing;
  identical reruns do not rewrite Bronze, changed bytes are refused.
- tests/test_ingest_boundaries.py: 9 synthetic cases.
- Docs: data contract section, naming keys, task specs §7 findings,
  architecture, README, progress. Workbook: ID 4/11 descriptions and risk
  row 9 rewritten to the pre-merger scope (original wording quoted); ID 4
  Đang làm 90%.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Phan_cong_cong_viec_DW_khi_tuong.xlsx
+++ b/Phan_cong_cong_viec_DW_khi_tuong.xlsx
@@ -2101,8 +2101,10 @@
       <c r="E8" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="F8" s="20" t="s">
-        <v>70</v>
+      <c r="F8" s="20" t="inlineStr">
+        <is>
+          <t>Tải GeoJSON địa giới Việt Nam, ranh giới TRƯỚC sáp nhập (63 tỉnh). Đổi phạm vi ngày 21/10/2026; mô tả gốc: "ranh giới sau sáp nhập 1/7/2025"</t>
+        </is>
       </c>
       <c r="G8" s="19" t="s">
         <v>14</v>
@@ -2123,15 +2125,17 @@
         <f aca="false">'Tổng quan'!$E$11+(C8-1)*7+4</f>
         <v>46311</v>
       </c>
-      <c r="M8" s="22" t="s">
-        <v>62</v>
+      <c r="M8" s="22" t="inlineStr">
+        <is>
+          <t>Đang làm</t>
+        </is>
       </c>
       <c r="N8" s="23" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="O8" s="24" t="inlineStr">
         <is>
-          <t>22/10: chưa bắt đầu, trễ hạn tuần 1. Phạm vi đã chốt 21/10 (N2): dùng ranh giới trước sáp nhập (63 tỉnh), không làm ranh giới sau 1/7/2025, vì giai đoạn nghiên cứu gần như toàn bộ trước sáp nhập. Nguồn ứng viên và tiêu chí: docs/task-specs-weeks-2-5.md §7</t>
+          <t>22/10: scripts/ingest_boundaries.py: GeoJSON 63 tỉnh trước sáp nhập (geoBoundaries VNM ADM1, commit 9469f09, năm 2008) trong Bronze kèm manifest (SHA-256, giấy phép, CRS); Silver 25 tỉnh miền Bắc (QĐ 368, 369/QĐ-TTg), 8 tỉnh có dữ liệu. Hình học hợp lệ 64/64; 8/8 điểm nằm đúng tỉnh trong dim_location. Hạn chế: ranh giới lấy từ Wikipedia/Wikimedia, độ chi tiết thấp; giấy phép ghi Public Domain (geoBoundaries) và ODbL (HDX). Phạm vi đã chốt 21/10: không làm ranh giới sau sáp nhập</t>
         </is>
       </c>
     </row>
@@ -2461,8 +2465,10 @@
       <c r="E15" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="F15" s="20" t="s">
-        <v>87</v>
+      <c r="F15" s="20" t="inlineStr">
+        <is>
+          <t>DimLocation (chỉ tỉnh trước sáp nhập; mô tả gốc "tỉnh cũ + tỉnh mới", đổi ngày 21/10/2026), DimStation, gán trạm theo khoảng cách bằng GeoPandas</t>
+        </is>
       </c>
       <c r="G15" s="19" t="s">
         <v>14</v>
@@ -2493,7 +2499,7 @@
       </c>
       <c r="O15" s="24" t="inlineStr">
         <is>
-          <t>21/10: mã/tọa độ trạm đã xác minh (Meteostat + NOAA ISD). Hợp lệ: HAN 48820, HPH 48826, TNG 48831, LCA 48803; dim_station 12 trạm (thêm 48823 Nam Định cho mưa ngày). 22/10: 48820 = sân bay Nội Bài (22,0 km, vai trò nearest_available); thêm station_role, distance_km (sql/05). Khoảng cách tính bằng haversine, không dùng GeoPandas. Tỉnh: đã chốt 21/10 chỉ dùng tỉnh trước sáp nhập, không làm ánh xạ tỉnh cũ-mới</t>
+          <t>21/10: mã/tọa độ trạm đã xác minh (Meteostat + NOAA ISD). Hợp lệ: HAN 48820, HPH 48826, TNG 48831, LCA 48803; dim_station 12 trạm (thêm 48823 Nam Định cho mưa ngày). 22/10: 48820 = sân bay Nội Bài (22,0 km, vai trò nearest_available); thêm station_role, distance_km (sql/05). Khoảng cách tính bằng haversine, không dùng GeoPandas. Tỉnh: chỉ dùng tỉnh trước sáp nhập (đã chốt 21/10); 8 điểm đã kiểm tra nằm đúng tỉnh trên GeoJSON ID 4 (22/10)</t>
         </is>
       </c>
     </row>
@@ -4226,8 +4232,10 @@
       <c r="B9" s="20" t="s">
         <v>205</v>
       </c>
-      <c r="C9" s="20" t="s">
-        <v>206</v>
+      <c r="C9" s="20" t="inlineStr">
+        <is>
+          <t>Địa điểm = điểm tọa độ; DimLocation chỉ lưu tỉnh trước sáp nhập; GeoJSON dùng ranh giới trước sáp nhập (63 tỉnh). Đổi ngày 21/10/2026; cách xử lý gốc: "DimLocation lưu cả tỉnh cũ và mới; GeoJSON dùng ranh giới mới"</t>
+        </is>
       </c>
       <c r="D9" s="19" t="s">
         <v>14</v>

</xml_diff>

<commit_message>
feat: complete week-1 tasks (IDs 1, 2, 3, 5, 8, 14)
- ID 1: Airflow webserver/scheduler verified end-to-end (health DAG run).
- ID 3: star schema diagram generated from the live catalog
  (docs/diagrams/star-schema.md).
- IDs 2/8: Open-Meteo Bronze keeps the received bytes with a manifest
  (request, SHA-256, coverage, response metadata); skips by manifest
  checksum instead of size; --replace-legacy replaces old objects only
  when hourly data are identical (all 80 replaced). Silver verifies the
  manifest checksum.
- IDs 5/14: scripts/ingest_era5.py requests ERA5 monthly from the CDS,
  checks NetCDF (or the zip of instant/accum NetCDF the CDS returns),
  stores it unchanged with a manifest incl. the job id; 2024-01 loaded.
  cdsapi 0.7.7 added to the lock; CDS credentials come from .env.
- Docs, progress, workbook updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Phan_cong_cong_viec_DW_khi_tuong.xlsx
+++ b/Phan_cong_cong_viec_DW_khi_tuong.xlsx
@@ -1971,11 +1971,11 @@
         </is>
       </c>
       <c r="N5" s="23" t="n">
-        <v>80</v>
+        <v>95</v>
       </c>
       <c r="O5" s="24" t="inlineStr">
         <is>
-          <t>Compose/Dockerfile build OK; MinIO+Postgres đã chạy. Chưa kiểm chứng webserver/scheduler end-to-end (21/10)</t>
+          <t>22/10: kiểm chứng đầu-cuối: webserver + scheduler healthy (/health), 2 DAG nạp không lỗi, DAG kiểm tra hệ thống chạy thành công qua REST API (cả 2 task); DW giữ nguyên sau khi khởi động lại. Kiểm chứng trên 1 máy (cả nhóm hiện là 1 người). Đủ tiêu chí, chờ bạn xác nhận Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2023,11 +2023,11 @@
         </is>
       </c>
       <c r="N6" s="23" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="O6" s="24" t="inlineStr">
         <is>
-          <t>Đã có 3 bucket và key đúng quy ước. Còn thiếu: Bronze chưa giữ nguyên payload gốc (_pipeline_metadata)</t>
+          <t>22/10: 3 bucket, key đúng quy ước. Bronze Open-Meteo giữ nguyên bytes gốc + manifest (SHA-256, độ phủ, tọa độ lưới) cho cả 80 file; bỏ qua theo checksum, không theo kích thước. Còn lại: Bronze Meteostat chưa có manifest (thuộc ID 9)</t>
         </is>
       </c>
     </row>
@@ -2077,11 +2077,11 @@
         </is>
       </c>
       <c r="N7" s="23" t="n">
-        <v>80</v>
+        <v>95</v>
       </c>
       <c r="O7" s="24" t="inlineStr">
         <is>
-          <t>22/10: DDL + sơ đồ star schema (outputs/dfd-weather-20261013, chỉ có trên máy cục bộ vì outputs/ không đưa lên Git). Đã chốt: cơ sở lịch UTC+7; prediction (sql/04, sql/05). Còn mở: nhiều trạm/nguồn trên cùng điểm</t>
+          <t>22/10: sơ đồ Star Schema sinh từ DW thật (9 bảng, 14 khóa ngoại, grain từng fact): docs/diagrams/star-schema.md; thay bản phác 13/10 chỉ có trong outputs/. Cơ sở lịch UTC+7, prediction, chọn trạm (tối đa 1 trạm/điểm) đều đã chốt. Chờ bạn xác nhận Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2177,15 +2177,17 @@
         <f aca="false">'Tổng quan'!$E$11+(C9-1)*7+4</f>
         <v>46311</v>
       </c>
-      <c r="M9" s="22" t="s">
-        <v>62</v>
+      <c r="M9" s="22" t="inlineStr">
+        <is>
+          <t>Đang làm</t>
+        </is>
       </c>
       <c r="N9" s="23" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="O9" s="24" t="inlineStr">
         <is>
-          <t>22/10: chưa bắt đầu, trễ hạn tuần 1. Phạm vi đã thống nhất 22/10 (N1/N2, chờ N3 xác nhận): ERA5 hourly single levels, vùng 19,5–23,5°N, 102,5–107,5°E, biến t2m, d2m, tp, sp, u10, v10, tcc, 2016–2025, NetCDF. Việc cần N3: tạo tài khoản Copernicus CDS và chấp nhận giấy phép; chưa tải khi chưa có tài khoản</t>
+          <t>22/10: đã đăng ký CDS, chấp nhận giấy phép ERA5; yêu cầu đầu tiên chạy thành công (job 70c1b649…, xếp hàng 80 s, xử lý ~6,5 phút). Bronze có tháng 1/2024: era5_north_vietnam_hourly_202401.zip (3,8 MB, 2 file NetCDF: 6 biến tức thời + lượng mưa tp; 744 giờ; lưới 17×23 ô) kèm manifest. Chưa gửi 119 tháng còn lại của 2016–2025 (chờ bạn đồng ý)</t>
         </is>
       </c>
     </row>
@@ -2337,11 +2339,11 @@
         </is>
       </c>
       <c r="N12" s="23" t="n">
-        <v>80</v>
+        <v>95</v>
       </c>
       <c r="O12" s="24" t="inlineStr">
         <is>
-          <t>21/10: chạy lại trên máy N1/N2: 80/80 file Bronze (8 điểm × 2016–2025), 326 s; «0 lỗi» dựa trên số object vì script khi đó vẫn thoát mã 0 khi có file lỗi. 22/10: đã sửa: file lỗi → thoát mã 1 sau khi thử hết các file còn lại, chỉ thử lại lỗi 429/5xx/mạng; Silver coi file Bronze thiếu là lỗi. Còn lệch: Bronze chưa giữ nguyên payload gốc, thiếu manifest</t>
+          <t>22/10: Bronze giữ nguyên payload gốc + manifest; tải lại 80/80 file (339 s, 0 lỗi), dữ liệu theo giờ giống hệt bản cũ; Silver 2024 giống từng dòng (70.272). Chạy lại: bỏ qua 80 file theo checksum. Lỗi thoát mã 1 (sửa 22/10). Tiêu chí «SHA bằng bản tải mới» không đạt được về nguyên tắc vì phản hồi có generationtime_ms; thay bằng so sánh dữ liệu theo giờ</t>
         </is>
       </c>
     </row>
@@ -2645,13 +2647,19 @@
         <f aca="false">'Tổng quan'!$E$11+(C18-1)*7+4</f>
         <v>46325</v>
       </c>
-      <c r="M18" s="22" t="s">
-        <v>62</v>
+      <c r="M18" s="22" t="inlineStr">
+        <is>
+          <t>Đang làm</t>
+        </is>
       </c>
       <c r="N18" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O18" s="24"/>
+        <v>60</v>
+      </c>
+      <c r="O18" s="24" t="inlineStr">
+        <is>
+          <t>22/10: scripts/ingest_era5.py đọc NetCDF bằng xarray để kiểm tra (biến, số giờ, vùng) rồi lưu Bronze nguyên bản kèm manifest; đã chạy thật cho 2024-01 (khớp yêu cầu, chạy lại bỏ qua theo checksum). Còn lại: các tháng khác</t>
+        </is>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="19" t="n">

</xml_diff>

<commit_message>
feat(airflow): Bronze -> DW pipeline DAG with reconciliation (ID 17); docs sweep
- dags/dag_weather_pipeline.py: validate window -> ingest Open-Meteo and
  Meteostat -> Silver -> seed dimensions -> Gold/DW -> reconcile; year
  window 2016-2025 and optional location; manual, one run at a time;
  ingestion retries once.
- scripts/reconcile_dw.py: DW vs Silver row counts per source x location x
  UTC year; any difference fails and is reported in gold/quality_reports.
- Real runs on 2024: HAN, rerun without new rows, forced MinIO outage then
  resume of the same run, all 8 locations (79,039 = 79,039).
- Documentation brought up to date with the 2026-10-22 work; ID 17 test
  window decided as one year x one location.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Phan_cong_cong_viec_DW_khi_tuong.xlsx
+++ b/Phan_cong_cong_viec_DW_khi_tuong.xlsx
@@ -2447,7 +2447,7 @@
       </c>
       <c r="O14" s="24" t="inlineStr">
         <is>
-          <t>21/10: Silver chạy lại: Open-Meteo 701.376 dòng; Meteostat 87.485 dòng sau khi loại 436.502 giá trị mô hình và 43.575 dòng không có quan trắc; 60 file Silver cũ đã xóa; 0 xung đột, 0 lỗi</t>
+          <t>21/10: Silver chạy lại: Open-Meteo 701.376 dòng; Meteostat 87.485 dòng sau khi loại 436.502 giá trị mô hình và 43.575 dòng không có quan trắc; 60 file Silver cũ đã xóa; 0 xung đột, 0 lỗi. 22/10: file Bronze Open-Meteo bị thiếu tính là lỗi (trừ khi có --allow-missing); Silver kiểm tra SHA-256 của Bronze theo manifest; chạy lại Silver 2024 giống từng dòng (70.272)</t>
         </is>
       </c>
     </row>
@@ -2755,7 +2755,7 @@
       </c>
       <c r="O20" s="24" t="inlineStr">
         <is>
-          <t>21/10: Gold 2016–2025 nạp lại trên máy N1/N2, 120 tháng, 0 lỗi: 832.436 dòng (233 s) trước khi lọc Meteostat, sau đó 788.861 dòng (292 s). 22/10: station_key trong Gold lưu dạng số nguyên (đã áp dụng cho 2024; các năm khác khi nạp lại). Bộ đặc trưng ML nằm ở gold/ml_features (ID 23); chưa có bảng pivot đa nguồn</t>
+          <t>21/10: Gold 2016–2025 nạp lại trên máy N1/N2, 120 tháng, 0 lỗi: 832.436 dòng (233 s) trước khi lọc Meteostat, sau đó 788.861 dòng (292 s). 22/10: nạp lại toàn bộ 2016–2025 (176 s, 0 lỗi, DW không đổi): cả 120 file Gold lưu station_key dạng số nguyên. Bộ đặc trưng ML nằm ở gold/ml_features (ID 23); chưa có bảng pivot đa nguồn</t>
         </is>
       </c>
     </row>
@@ -2799,13 +2799,19 @@
         <f aca="false">'Tổng quan'!$E$11+(C21-1)*7+4</f>
         <v>46339</v>
       </c>
-      <c r="M21" s="22" t="s">
-        <v>62</v>
+      <c r="M21" s="22" t="inlineStr">
+        <is>
+          <t>Đang làm</t>
+        </is>
       </c>
       <c r="N21" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O21" s="24"/>
+        <v>90</v>
+      </c>
+      <c r="O21" s="24" t="inlineStr">
+        <is>
+          <t>22/10: dags/dag_weather_pipeline.py (weather_bronze_to_dw_dag): tải Open-Meteo + Meteostat → Silver → seed dim → Gold → DW → đối chiếu số dòng DW với Silver (scripts/reconcile_dw.py). Tham số năm 2016–2025 và điểm; chạy tay, 1 lượt một lúc. Đã chạy thật: 2024 HAN (khớp 17.551 dòng), chạy lại không thêm dòng, cố ý tắt MinIO → lỗi rõ ràng rồi chạy tiếp thành công, 2024 cả 8 điểm (khớp 79.039 dòng). Lệch so với đặc tả: cửa sổ nhỏ nhất là 1 năm (script theo năm), chưa gồm GHCNh/ERA5</t>
+        </is>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="19" t="n">

</xml_diff>

<commit_message>
feat(airflow): add GHCNh daily rain to the pipeline DAG; 2016-2025 run (ID 17)
- GHCNh scripts accept --location (stations resolved from station_config;
  a location without a station is a no-op).
- DAG: ingest_ghcnh -> transform_ghcnh_to_silver -> load_station_daily_rain.
- reconcile_dw also compares daily rain per station x year.
- Acceptance run 2016-2025, all locations: no downloads, 3 min 43 s,
  788,861 = 788,861 hourly rows and 17,866 = 17,866 station-days.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Phan_cong_cong_viec_DW_khi_tuong.xlsx
+++ b/Phan_cong_cong_viec_DW_khi_tuong.xlsx
@@ -2805,11 +2805,11 @@
         </is>
       </c>
       <c r="N21" s="23" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="O21" s="24" t="inlineStr">
         <is>
-          <t>22/10: dags/dag_weather_pipeline.py (weather_bronze_to_dw_dag): tải Open-Meteo + Meteostat → Silver → seed dim → Gold → DW → đối chiếu số dòng DW với Silver (scripts/reconcile_dw.py). Tham số năm 2016–2025 và điểm; chạy tay, 1 lượt một lúc. Đã chạy thật: 2024 HAN (khớp 17.551 dòng), chạy lại không thêm dòng, cố ý tắt MinIO → lỗi rõ ràng rồi chạy tiếp thành công, 2024 cả 8 điểm (khớp 79.039 dòng). Lệch so với đặc tả: cửa sổ nhỏ nhất là 1 năm (script theo năm), chưa gồm GHCNh/ERA5</t>
+          <t>22/10: dags/dag_weather_pipeline.py (weather_bronze_to_dw_dag): Open-Meteo, Meteostat, mưa ngày GHCNh: tải → Silver → seed dim → Gold/DW → đối chiếu DW với Silver (scripts/reconcile_dw.py). Tham số năm 2016–2025 và điểm; chạy tay, 1 lượt một lúc. Đã chạy: 2024 HAN, chạy lại không thêm dòng, cố ý tắt MinIO rồi chạy tiếp thành công, 2024 cả 8 điểm, và cả 2016–2025 (3 phút 43 giây; khớp 788.861 dòng giờ và 17.866 ngày mưa; không tải lại gì). Cửa sổ nhỏ nhất 1 năm × 1 điểm (đã chốt). Chờ bạn xác nhận Hoàn thành</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(workbook): ID 24 status; refresh ERA5 and Recall notes (IDs 5, 14, 28, risk 4)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Phan_cong_cong_viec_DW_khi_tuong.xlsx
+++ b/Phan_cong_cong_viec_DW_khi_tuong.xlsx
@@ -2187,7 +2187,7 @@
       </c>
       <c r="O9" s="24" t="inlineStr">
         <is>
-          <t>22/10: đã đăng ký CDS, chấp nhận giấy phép ERA5; yêu cầu đầu tiên chạy thành công (job 70c1b649…, xếp hàng 80 s, xử lý ~6,5 phút). Bronze có tháng 1/2024: era5_north_vietnam_hourly_202401.zip (3,8 MB, 2 file NetCDF: 6 biến tức thời + lượng mưa tp; 744 giờ; lưới 17×23 ô) kèm manifest. Chưa gửi 119 tháng còn lại của 2016–2025 (chờ bạn đồng ý)</t>
+          <t>22/10: đã đăng ký CDS, chấp nhận giấy phép ERA5; yêu cầu đầu tiên chạy thành công (job 70c1b649…, ~6,5 phút). Đã gửi yêu cầu cho 2016–2025, lần lượt từng tháng (CDS từ chối gửi nhiều yêu cầu cùng lúc). Đầu ra «yêu cầu tải đã vào hàng đợi» đã đạt; tải đủ file thuộc ID 14</t>
         </is>
       </c>
     </row>
@@ -2657,7 +2657,7 @@
       </c>
       <c r="O18" s="24" t="inlineStr">
         <is>
-          <t>22/10: scripts/ingest_era5.py đọc NetCDF bằng xarray để kiểm tra (biến, số giờ, vùng) rồi lưu Bronze nguyên bản kèm manifest; đã chạy thật cho 2024-01 (khớp yêu cầu, chạy lại bỏ qua theo checksum). Còn lại: các tháng khác</t>
+          <t>22/10: scripts/ingest_era5.py đọc NetCDF bằng xarray để kiểm tra (biến, số giờ, vùng) rồi lưu Bronze nguyên bản kèm manifest; chạy lại bỏ qua theo checksum. Bronze có 2016-01, 2016-02, 2024-01. Đang tải lần lượt: 2024–2025 trước (phạm vi dự phòng, business-requirements §5a), rồi 2016–2023. CDS chỉ cho 1 yêu cầu chờ mỗi lúc; một tháng chờ hàng đợi ~1 giờ 40 phút, xử lý ~4 phút, nên cần vài ngày</t>
         </is>
       </c>
     </row>
@@ -3163,13 +3163,19 @@
         <f aca="false">'Tổng quan'!$E$11+(C28-1)*7+4</f>
         <v>46353</v>
       </c>
-      <c r="M28" s="22" t="s">
-        <v>62</v>
+      <c r="M28" s="22" t="inlineStr">
+        <is>
+          <t>Đang làm</t>
+        </is>
       </c>
       <c r="N28" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O28" s="24"/>
+        <v>95</v>
+      </c>
+      <c r="O28" s="24" t="inlineStr">
+        <is>
+          <t>22/10: scripts/quality_gate.py, task quality_gate trong DAG (sau bước Silver, trước khi ghi DW). Dừng DAG khi: thiếu cột hoặc khóa trống; giờ không UTC hoặc sai tháng; trùng nguồn × điểm × giờ; giá trị ngoài khoảng hợp lệ của data-contract; thiếu giờ Open-Meteo; GHCNh trùng ngày, sai khung 12:00 UTC, mưa ngoài 0–999 mm. Cảnh báo, không dừng (ngưỡng chốt 22/10 từ dữ liệu 2016–2025): độ phủ Meteostat &lt; 95%, GHCNh &lt; 90%; Open-Meteo thiếu giá trị; Meteostat thiếu nhiệt độ/độ ẩm &gt; 5%; nhiệt độ ngoài 0–45 °C; áp suất ngoài 950–1050 hPa; mưa giờ &gt; 100 mm; mưa ngày ≥ 300 mm chưa duyệt. Dữ liệu thật 2016–2025: 712 kiểm tra, 0 lỗi, 0 cảnh báo; DAG 2024 HAN 12/12 task; test tích hợp xác nhận task Airflow báo lỗi khi Silver sai. Chờ bạn xác nhận Hoàn thành</t>
+        </is>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="19" t="n">
@@ -3359,7 +3365,7 @@
       </c>
       <c r="O32" s="24" t="inlineStr">
         <is>
-          <t>21/10: gold/ml_models/cart_rain_next24h_v1 (model.joblib + report.json). Lưới 120 cấu hình, chọn trên validation 2024: max_depth=8, min_samples_leaf=50, class_weight=balanced, ccp_alpha=1e-4, 88 lá, ngưỡng 0,40. Validation (nhãn đã sửa 22/10): Precision 0,760 / Recall 0,819 / F1 0,789. Model train trên nhãn v1 (0,73% sai), không train lại để giữ test độc lập. 22/10: chặn ghi đè model (model đã chấm test thì không cho ghi đè). Chọn cấu hình và ngưỡng theo F1, chưa có quy tắc ưu tiên Recall (đề xuất chờ duyệt). Do N1/N2 làm thay N3</t>
+          <t>21/10: gold/ml_models/cart_rain_next24h_v1 (model.joblib + report.json). Lưới 120 cấu hình, chọn trên validation 2024: max_depth=8, min_samples_leaf=50, class_weight=balanced, ccp_alpha=1e-4, 88 lá, ngưỡng 0,40. Validation (nhãn đã sửa 22/10): Precision 0,760 / Recall 0,819 / F1 0,789. Model train trên nhãn v1 (0,73% sai), không train lại để giữ test độc lập. 22/10: chặn ghi đè model (model đã chấm test thì không cho ghi đè). Chọn cấu hình và ngưỡng theo F1. Quy tắc ưu tiên Recall đã chốt 22/10: ngưỡng 0,36 (Recall validation 0,88); 0,40 vẫn là kết quả test chính thức. Chờ N3 duyệt (rain-label.md). Do N1/N2 làm thay N3</t>
         </is>
       </c>
     </row>
@@ -4159,7 +4165,7 @@
       </c>
       <c r="F4" s="24" t="inlineStr">
         <is>
-          <t>22/10: ID 5 chưa bắt đầu; đề xuất phạm vi và thứ tự ở docs/business-requirements.md §5a</t>
+          <t>22/10: đã đăng ký CDS, chấp nhận giấy phép, tải theo tháng. Thực tế: một tháng chờ hàng đợi ~1 giờ 40 phút; CDS từ chối gửi nhiều yêu cầu cùng lúc. Đang tải 2024–2025 trước rồi 2016–2023, cần vài ngày (ID 5, 14)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(dw): load ERA5 into the DW and add the ERA5 chain to the DAG (IDs 16-18, 24)
- Gold loader, quality gate, and reconciliation read era5/weather_hourly/ as well;
  ERA5 is a complete-hours source; a missing ERA5 location-month fails the month.
- Gate: ERA5 missing-value warnings and its own pressure limit (900-1050 hPa,
  grid-cell terrain; observed minimum 916.89 hPa at LCA).
- DAG: ingest_era5_timeseries -> transform_era5_to_silver -> quality_gate.
- ERA5 time-series ingestion creates the CDS client only when it must download.
- 2016-2025 DAG run: 14/14 tasks after recreating the Airflow containers with the
  CDS environment and resuming the failed task; DW 1,490,237 rows (ERA5 701,376),
  reconciliation equal, gate 1,032 checks with 0 failures and 0 warnings.
- Docs, progress, and workbook notes; Power BI guide reference rows for ERA5.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Phan_cong_cong_viec_DW_khi_tuong.xlsx
+++ b/Phan_cong_cong_viec_DW_khi_tuong.xlsx
@@ -2761,7 +2761,7 @@
       </c>
       <c r="O20" s="24" t="inlineStr">
         <is>
-          <t>21/10: Gold 2016–2025 nạp lại trên máy N1/N2, 120 tháng, 0 lỗi: 832.436 dòng (233 s) trước khi lọc Meteostat, sau đó 788.861 dòng (292 s). 22/10: nạp lại toàn bộ 2016–2025 (176 s, 0 lỗi, DW không đổi): cả 120 file Gold lưu station_key dạng số nguyên. Bộ đặc trưng ML nằm ở gold/ml_features (ID 23); chưa có bảng pivot đa nguồn</t>
+          <t>21/10: Gold 2016–2025 nạp lại trên máy N1/N2, 120 tháng, 0 lỗi: 832.436 dòng (233 s) trước khi lọc Meteostat, sau đó 788.861 dòng (292 s). 22/10: nạp lại toàn bộ 2016–2025 (176 s, 0 lỗi, DW không đổi): cả 120 file Gold lưu station_key dạng số nguyên. Bộ đặc trưng ML nằm ở gold/ml_features (ID 23); chưa có bảng pivot đa nguồn 23/10: Gold mỗi tháng gồm cả ERA5 (3 nguồn: Open-Meteo, Meteostat, ERA5). Chưa có bảng pivot đa nguồn cho ML.</t>
         </is>
       </c>
     </row>
@@ -2815,7 +2815,7 @@
       </c>
       <c r="O21" s="24" t="inlineStr">
         <is>
-          <t>22/10: dags/dag_weather_pipeline.py (weather_bronze_to_dw_dag): Open-Meteo, Meteostat, mưa ngày GHCNh: tải → Silver → seed dim → Gold/DW → đối chiếu DW với Silver (scripts/reconcile_dw.py). Tham số năm 2016–2025 và điểm; chạy tay, 1 lượt một lúc. Đã chạy: 2024 HAN, chạy lại không thêm dòng, cố ý tắt MinIO rồi chạy tiếp thành công, 2024 cả 8 điểm, và cả 2016–2025 (3 phút 43 giây; khớp 788.861 dòng giờ và 17.866 ngày mưa; không tải lại gì). Cửa sổ nhỏ nhất 1 năm × 1 điểm (đã chốt). Chờ bạn xác nhận Hoàn thành</t>
+          <t>22/10: dags/dag_weather_pipeline.py (weather_bronze_to_dw_dag): Open-Meteo, Meteostat, mưa ngày GHCNh: tải → Silver → seed dim → Gold/DW → đối chiếu DW với Silver (scripts/reconcile_dw.py). Tham số năm 2016–2025 và điểm; chạy tay, 1 lượt một lúc. Đã chạy: 2024 HAN, chạy lại không thêm dòng, cố ý tắt MinIO rồi chạy tiếp thành công, 2024 cả 8 điểm, và cả 2016–2025 (3 phút 43 giây; khớp 788.861 dòng giờ và 17.866 ngày mưa; không tải lại gì). Cửa sổ nhỏ nhất 1 năm × 1 điểm (đã chốt). Chờ bạn xác nhận Hoàn thành 23/10: thêm nhánh ERA5 (tải time-series → Silver) trước bước quality_gate. Chạy 2016–2025: 14/14 task thành công (lần đầu bước ERA5 lỗi vì container Airflow chưa có khóa CDS; đã sửa, chạy tiếp từ bước lỗi); đối chiếu 1.490.237 = 1.490.237 dòng giờ, 17.866 = 17.866 ngày mưa.</t>
         </is>
       </c>
     </row>
@@ -2867,7 +2867,7 @@
       </c>
       <c r="O22" s="24" t="inlineStr">
         <is>
-          <t>21/10: DW sạch: 788.861 dòng (Open-Meteo 701.376 + Meteostat HAN 87.485), 0 trùng khóa; rút dòng sai đã kiểm chứng trên dữ liệu thật; lần nạp cuối 292 s (bản trước ghi 3.493 s là sai). 22/10: phạm vi xóa khi nạp lại tính theo phạm vi yêu cầu (nguồn biến mất bị xóa; thiếu file Silver Open-Meteo của một vị trí thì tháng đó báo lỗi); thêm pressure_type (sql/05). Chạy lại 2024 trên trạng thái hiện tại: 79.039 dòng, không đổi. Bản 994.145 dòng trên máy bacnx đã lỗi thời</t>
+          <t>21/10: DW sạch: 788.861 dòng (Open-Meteo 701.376 + Meteostat HAN 87.485), 0 trùng khóa; rút dòng sai đã kiểm chứng trên dữ liệu thật; lần nạp cuối 292 s (bản trước ghi 3.493 s là sai). 22/10: phạm vi xóa khi nạp lại tính theo phạm vi yêu cầu (nguồn biến mất bị xóa; thiếu file Silver Open-Meteo của một vị trí thì tháng đó báo lỗi); thêm pressure_type (sql/05). Chạy lại 2024 trên trạng thái hiện tại: 79.039 dòng, không đổi. Bản 994.145 dòng trên máy bacnx đã lỗi thời 23/10: nạp thêm ERA5 701.376 dòng (đã chốt nạp ERA5 theo đề cương §8, §10); DW 1.490.237 dòng, 0 trùng khóa; Open-Meteo, Meteostat, mưa ngày, dự báo không đổi.</t>
         </is>
       </c>
     </row>
@@ -3179,7 +3179,7 @@
       </c>
       <c r="O28" s="24" t="inlineStr">
         <is>
-          <t>22/10: scripts/quality_gate.py, task quality_gate trong DAG (sau bước Silver, trước khi ghi DW). Dừng DAG khi: thiếu cột hoặc khóa trống; giờ không UTC hoặc sai tháng; trùng nguồn × điểm × giờ; giá trị ngoài khoảng hợp lệ của data-contract; thiếu giờ Open-Meteo; GHCNh trùng ngày, sai khung 12:00 UTC, mưa ngoài 0–999 mm. Cảnh báo, không dừng (ngưỡng chốt 22/10 từ dữ liệu 2016–2025): độ phủ Meteostat &lt; 95%, GHCNh &lt; 90%; Open-Meteo thiếu giá trị; Meteostat thiếu nhiệt độ/độ ẩm &gt; 5%; nhiệt độ ngoài 0–45 °C; áp suất ngoài 950–1050 hPa; mưa giờ &gt; 100 mm; mưa ngày ≥ 300 mm chưa duyệt. Dữ liệu thật 2016–2025: 712 kiểm tra, 0 lỗi, 0 cảnh báo; DAG 2024 HAN 12/12 task; test tích hợp xác nhận task Airflow báo lỗi khi Silver sai. Chờ bạn xác nhận Hoàn thành</t>
+          <t>22/10: scripts/quality_gate.py, task quality_gate trong DAG (sau bước Silver, trước khi ghi DW). Dừng DAG khi: thiếu cột hoặc khóa trống; giờ không UTC hoặc sai tháng; trùng nguồn × điểm × giờ; giá trị ngoài khoảng hợp lệ của data-contract; thiếu giờ Open-Meteo; GHCNh trùng ngày, sai khung 12:00 UTC, mưa ngoài 0–999 mm. Cảnh báo, không dừng (ngưỡng chốt 22/10 từ dữ liệu 2016–2025): độ phủ Meteostat &lt; 95%, GHCNh &lt; 90%; Open-Meteo thiếu giá trị; Meteostat thiếu nhiệt độ/độ ẩm &gt; 5%; nhiệt độ ngoài 0–45 °C; áp suất ngoài 950–1050 hPa; mưa giờ &gt; 100 mm; mưa ngày ≥ 300 mm chưa duyệt. Dữ liệu thật 2016–2025: 712 kiểm tra, 0 lỗi, 0 cảnh báo; DAG 2024 HAN 12/12 task; test tích hợp xác nhận task Airflow báo lỗi khi Silver sai. Chờ bạn xác nhận Hoàn thành 23/10: kiểm tra cả ERA5 (bắt buộc đủ giờ; cảnh báo áp suất ngoài 900–1050 hPa vì ô lưới cao hơn điểm): 1.032 kiểm tra, 0 lỗi, 0 cảnh báo.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(ml): threshold comparison and error analysis of CART v1 (ID 36)
Validation scan on the model's threshold grid with the F1 and Recall rules
(0.40 and 0.36); test 2025 only at predeclared thresholds, disclosed as
post-hoc; error breakdowns by rain amount, near-threshold false alarms, rain
before the origin, season, location, period, and calibration.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Phan_cong_cong_viec_DW_khi_tuong.xlsx
+++ b/Phan_cong_cong_viec_DW_khi_tuong.xlsx
@@ -3759,13 +3759,19 @@
         <f aca="false">'Tổng quan'!$E$11+(C40-1)*7+4</f>
         <v>46367</v>
       </c>
-      <c r="M40" s="22" t="s">
-        <v>62</v>
+      <c r="M40" s="22" t="inlineStr">
+        <is>
+          <t>Đang làm</t>
+        </is>
       </c>
       <c r="N40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O40" s="24"/>
+        <v>95</v>
+      </c>
+      <c r="O40" s="24" t="inlineStr">
+        <is>
+          <t>23/10: scripts/analyze_cart_thresholds.py → gold/ml_models/cart_rain_next24h_v1/threshold_error_analysis.json. So sánh ngưỡng trên validation 2024 (lưới 0,30–0,70 của quy tắc chọn ngưỡng): quy tắc F1 vẫn ra 0,40 (ngưỡng chính thức), quy tắc ưu tiên Recall ra 0,36. Test 2025 chỉ tính ở các ngưỡng đã chốt (phân tích sau, có ghi rõ): 0,40 → P 0,762 / R 0,792 / F1 0,777; 0,36 → 0,723 / 0,848 / 0,780 (thêm 2.709 báo động giả, bớt 1.945 ca bỏ sót). Lỗi: bỏ sót nhiều nhất ở mưa nhẹ 1–2 mm (42%); báo động giả phần lớn là cửa sổ có 0–1 mm; mưa sau 24 giờ khô chỉ bắt được 17%; mùa mưa F1 0,836, mùa khô 0,624. Chi tiết: rain-label.md. Do N1/N2 làm thay N3. Chờ bạn xác nhận Hoàn thành</t>
+        </is>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="19" t="n">

</xml_diff>

<commit_message>
feat(dw): query workload benchmark and performance findings (ID 26)
Read-only EXPLAIN ANALYZE benchmark of the dashboard refresh and reconciliation
queries; candidate indexes measured inside a rolled-back transaction did not
change the aggregate plans, so no index is added. Findings and the proposed
latency target are in warehouse-schema.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Phan_cong_cong_viec_DW_khi_tuong.xlsx
+++ b/Phan_cong_cong_viec_DW_khi_tuong.xlsx
@@ -3269,13 +3269,19 @@
         <f aca="false">'Tổng quan'!$E$11+(C30-1)*7+4</f>
         <v>46353</v>
       </c>
-      <c r="M30" s="22" t="s">
-        <v>62</v>
+      <c r="M30" s="22" t="inlineStr">
+        <is>
+          <t>Đang làm</t>
+        </is>
       </c>
       <c r="N30" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O30" s="24"/>
+        <v>90</v>
+      </c>
+      <c r="O30" s="24" t="inlineStr">
+        <is>
+          <t>23/10: đo thật bằng scripts/benchmark_dw_queries.py (EXPLAIN ANALYZE, 3 lần, trung vị) trên DW 1.490.237 dòng: nạp từng view cho dashboard 0,3–1,3 giây, tổng khoảng 5,8 giây; truy vấn đối chiếu 0,4 ms–1,2 giây. Index hiện có đã đủ cho truy vấn có lọc; đã thử thêm index ghép và index cho 4 khóa ngoại trong giao dịch rồi hoàn tác: không nhanh hơn (view tổng hợp phải quét cả bảng), nên không thêm. Đề xuất mục tiêu: mỗi view dưới 5 giây, truy vấn đối chiếu dưới 2 giây (đang đạt). Chờ bạn chốt mục tiêu</t>
+        </is>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="19" t="n">

</xml_diff>

<commit_message>
docs(dw): record the decided latency target for ID 26
The user accepted the proposed target on 2026-10-23: each view refresh
under 5 s and each reconciliation query under 2 s. The measured maxima
(1.3 s and 1.2 s) meet it without new indexes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Phan_cong_cong_viec_DW_khi_tuong.xlsx
+++ b/Phan_cong_cong_viec_DW_khi_tuong.xlsx
@@ -3275,11 +3275,11 @@
         </is>
       </c>
       <c r="N30" s="23" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="O30" s="24" t="inlineStr">
         <is>
-          <t>23/10: đo thật bằng scripts/benchmark_dw_queries.py (EXPLAIN ANALYZE, 3 lần, trung vị) trên DW 1.490.237 dòng: nạp từng view cho dashboard 0,3–1,3 giây, tổng khoảng 5,8 giây; truy vấn đối chiếu 0,4 ms–1,2 giây. Index hiện có đã đủ cho truy vấn có lọc; đã thử thêm index ghép và index cho 4 khóa ngoại trong giao dịch rồi hoàn tác: không nhanh hơn (view tổng hợp phải quét cả bảng), nên không thêm. Đề xuất mục tiêu: mỗi view dưới 5 giây, truy vấn đối chiếu dưới 2 giây (đang đạt). Chờ bạn chốt mục tiêu</t>
+          <t>23/10: đo thật bằng scripts/benchmark_dw_queries.py (EXPLAIN ANALYZE, 3 lần, trung vị) trên DW 1.490.237 dòng: nạp từng view cho dashboard 0,3–1,3 giây, tổng khoảng 5,8 giây; truy vấn đối chiếu 0,4 ms–1,2 giây. Index hiện có đã đủ cho truy vấn có lọc; đã thử thêm index ghép và index cho 4 khóa ngoại trong giao dịch rồi hoàn tác: không nhanh hơn (view tổng hợp phải quét cả bảng), nên không thêm. Mục tiêu đã chốt 23/10: mỗi view dưới 5 giây, truy vấn đối chiếu dưới 2 giây (đang đạt: tối đa 1,3 giây và 1,2 giây). Chờ bạn xác nhận Hoàn thành</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(ml): scoring DAG for CART RainNext24h with window-scoped publication (ID 32)
weather_rain_scoring_dag validates the window, scores the frozen model
with features recomputed from Silver, writes one Gold object per origin
day, publishes to the DW in one transaction, and checks DW against Gold.

- score_cart.py: artifact SHA-256 and feature-order checks; test origins
  only, targets inside 2016-2025; missing Silver or features fail
- publish_predictions.py: model must be in dim_model with the same
  artifact; rows update only when a value differs, so an unchanged rerun
  rewrites nothing; --dry-run and --check modes
- real run over 2025: 69,888 predictions, DW checksum unchanged

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Phan_cong_cong_viec_DW_khi_tuong.xlsx
+++ b/Phan_cong_cong_viec_DW_khi_tuong.xlsx
@@ -3579,13 +3579,19 @@
         <f aca="false">'Tổng quan'!$E$11+(C36-1)*7+4</f>
         <v>46360</v>
       </c>
-      <c r="M36" s="22" t="s">
-        <v>62</v>
+      <c r="M36" s="22" t="inlineStr">
+        <is>
+          <t>Đang làm</t>
+        </is>
       </c>
       <c r="N36" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O36" s="24"/>
+        <v>95</v>
+      </c>
+      <c r="O36" s="24" t="inlineStr">
+        <is>
+          <t>23/10: DAG weather_rain_scoring_dag (chạy tay): kiểm tra khoảng ngày → chấm điểm (scripts/score_cart.py: kiểm tra SHA-256 của mô hình, tính lại đặc trưng từ Silver, thiếu dữ liệu thì báo lỗi) → ghi Gold mỗi ngày một file → đăng lên DW (scripts/publish_predictions.py: chỉ ghi dòng thay đổi) → đối chiếu DW với Gold. Chỉ đăng dự báo tập test 2025 (01/01–30/12, mục tiêu không sang 2026). Chạy thật cả năm 2025: 4/4 task thành công trong 40 giây, 69.888 dự báo, DW không đổi dòng nào (mã băm trước và sau giống hệt); thử khoảng ngày sai thì DAG dừng ngay ở bước đầu. Chờ bạn xác nhận Hoàn thành</t>
+        </is>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="19" t="n">

</xml_diff>

<commit_message>
feat(airflow): watermark-driven incremental DAG (ID 25)
weather_incremental_dag runs daily, plans the next window of UTC years
from a watermark in Gold (new years plus a one-year lookback for late
corrections, never after 2025), triggers weather_bronze_to_dw_dag for it
and waits, and advances the watermark only after that run succeeded.

- pipeline_watermark.py: window rule, advance only from the planned base,
  set by hand with a recorded reason
- catchup off and paused at creation, so it never replays history alone
- real run: 2024-2025 replayed, watermark 2024 -> 2025, DW checksum
  unchanged; the next run skipped as up to date

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Phan_cong_cong_viec_DW_khi_tuong.xlsx
+++ b/Phan_cong_cong_viec_DW_khi_tuong.xlsx
@@ -3221,13 +3221,19 @@
         <f aca="false">'Tổng quan'!$E$11+(C29-1)*7+4</f>
         <v>46353</v>
       </c>
-      <c r="M29" s="22" t="s">
-        <v>62</v>
+      <c r="M29" s="22" t="inlineStr">
+        <is>
+          <t>Đang làm</t>
+        </is>
       </c>
       <c r="N29" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O29" s="24"/>
+        <v>95</v>
+      </c>
+      <c r="O29" s="24" t="inlineStr">
+        <is>
+          <t>23/10: DAG weather_incremental_dag chạy theo lịch hằng ngày (không chạy bù quá khứ, tạm dừng khi mới tạo): đọc mốc watermark trong MinIO (năm cuối đã nạp và đối chiếu xong) → chọn năm mới tiếp theo + chạy lại 1 năm trước để lấy dữ liệu sửa muộn, không vượt quá 2025 → gọi DAG Bronze→DW (task 17) và chờ → chỉ dời mốc khi lần chạy đó thành công. Chạy thật: đặt mốc 2024, lần chạy theo lịch xử lý 2024–2025 (14/14 task, 3 phút, đối chiếu 298.192 = 298.192 dòng giờ), mốc dời lên 2025; DW giống hệt trước khi chạy (không trùng, không đổi giá trị); lần chạy sau tự bỏ qua vì đã đủ đến 2025. Chờ bạn xác nhận Hoàn thành</t>
+        </is>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="19" t="n">

</xml_diff>

<commit_message>
feat(dw): station distances and nearest-station check with GeoPandas (ID 11)
assign_stations_geo.py projects the research points and stations to
UTM 48N, assigns the nearest station within 30 km with sjoin_nearest,
joins both to the pre-merger province polygons, and checks the station
registry and dim_station. Read-only; the DW is unchanged.

- GHCNh mapping equals the nearest station at all 8 points
- stored distances are spherical; the largest gap is 22.0 vs 21.86 km
- the Noi Bai coordinate falls 2.5 km inside Vinh Phuc on the polygon,
  reported as unresolved

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Phan_cong_cong_viec_DW_khi_tuong.xlsx
+++ b/Phan_cong_cong_viec_DW_khi_tuong.xlsx
@@ -2497,11 +2497,11 @@
         </is>
       </c>
       <c r="N15" s="23" t="n">
-        <v>60</v>
+        <v>95</v>
       </c>
       <c r="O15" s="24" t="inlineStr">
         <is>
-          <t>21/10: mã/tọa độ trạm đã xác minh (Meteostat + NOAA ISD). Hợp lệ: HAN 48820, HPH 48826, TNG 48831, LCA 48803; dim_station 12 trạm (thêm 48823 Nam Định cho mưa ngày). 22/10: 48820 = sân bay Nội Bài (22,0 km, vai trò nearest_available); thêm station_role, distance_km (sql/05). Khoảng cách tính bằng haversine, không dùng GeoPandas. Tỉnh: chỉ dùng tỉnh trước sáp nhập (đã chốt 21/10); 8 điểm đã kiểm tra nằm đúng tỉnh trên GeoJSON ID 4 (22/10)</t>
+          <t>21/10: mã/tọa độ trạm đã xác minh (Meteostat + NOAA ISD). Hợp lệ: HAN 48820, HPH 48826, TNG 48831, LCA 48803; dim_station 12 trạm (thêm 48823 Nam Định cho mưa ngày). 22/10: 48820 = sân bay Nội Bài (22,0 km, vai trò nearest_available); thêm station_role, distance_km (sql/05). Khoảng cách tính bằng haversine, không dùng GeoPandas. Tỉnh: chỉ dùng tỉnh trước sáp nhập (đã chốt 21/10); 8 điểm đã kiểm tra nằm đúng tỉnh trên GeoJSON ID 4 (22/10) 23/10: gán trạm bằng GeoPandas (scripts/assign_stations_geo.py): tính khoảng cách trên hệ tọa độ UTM 48N, trạm gần nhất trong 30 km, kiểm tra tỉnh của điểm và trạm, so với bảng trạm và dim_station (chỉ đọc). Kết quả đạt: trạm mưa GHCNh = trạm gần nhất ở cả 8 điểm; Meteostat HAN dùng Nội Bài (21,9 km) dù Hà Đông gần hơn (11,4 km, chưa chốt cho Meteostat); khoảng cách lưu lệch tối đa 0,14 km do tính trên hình cầu; 8/8 điểm đúng tỉnh. Tọa độ trạm Nội Bài nằm trong Vĩnh Phúc 2,5 km theo bản đồ geoBoundaries (chưa xác minh, không ảnh hưởng dữ liệu). DW không đổi. Chờ bạn xác nhận Hoàn thành</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(silver): keep the Open-Meteo grid cell and require a UTC payload (ID 10)
Open-Meteo Silver now carries grid_latitude, grid_longitude and
grid_elevation_m from the API response, and fails a payload whose
utc_offset_seconds is not 0 instead of shifting every hour.

- real run 2016-2025: 80 payloads at offset 0, previous columns
  identical in all 960 objects, gate and reconciliation passed, Gold
  reloaded, DW unchanged

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Phan_cong_cong_viec_DW_khi_tuong.xlsx
+++ b/Phan_cong_cong_viec_DW_khi_tuong.xlsx
@@ -2443,11 +2443,11 @@
         </is>
       </c>
       <c r="N14" s="23" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="O14" s="24" t="inlineStr">
         <is>
-          <t>21/10: Silver chạy lại: Open-Meteo 701.376 dòng; Meteostat 87.485 dòng sau khi loại 436.502 giá trị mô hình và 43.575 dòng không có quan trắc; 60 file Silver cũ đã xóa; 0 xung đột, 0 lỗi. 22/10: file Bronze Open-Meteo bị thiếu tính là lỗi (trừ khi có --allow-missing); Silver kiểm tra SHA-256 của Bronze theo manifest; chạy lại Silver 2024 giống từng dòng (70.272)</t>
+          <t>21/10: Silver chạy lại: Open-Meteo 701.376 dòng; Meteostat 87.485 dòng sau khi loại 436.502 giá trị mô hình và 43.575 dòng không có quan trắc; 60 file Silver cũ đã xóa; 0 xung đột, 0 lỗi. 22/10: file Bronze Open-Meteo bị thiếu tính là lỗi (trừ khi có --allow-missing); Silver kiểm tra SHA-256 của Bronze theo manifest; chạy lại Silver 2024 giống từng dòng (70.272) 23/10: Silver Open-Meteo lưu thêm tọa độ và độ cao ô lưới API trả về (grid_latitude, grid_longitude, grid_elevation_m) và báo lỗi nếu dữ liệu không ở UTC (utc_offset_seconds khác 0). Chạy lại 2016–2025: 80 file đều ở UTC, 701.376 dòng, các cột cũ giống hệt; quality gate 1.032 kiểm tra 0 lỗi; nạp lại Gold, đối chiếu 1.490.237 = 1.490.237; DW không đổi. Chờ bạn xác nhận Hoàn thành</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(gold): multi-source hourly pivot for ML (ID 16)
build_ml_pivot.py pivots the Gold observation months to one row per
location x UTC hour with one column per source and variable. Values are
never combined across sources and missing stays missing; the manifest
records units, pressure type per column, counts, and Gold SHA-256
lineage.

- checks before writing: unique key, per-source rows, per-variable
  counts and sums against Gold, per-source-year rows against the DW
- real run 2016-2025: 701,376 rows, all checks passed, DW unchanged
- also corrects the ID 10 progress note: Gold keeps only fact columns

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Phan_cong_cong_viec_DW_khi_tuong.xlsx
+++ b/Phan_cong_cong_viec_DW_khi_tuong.xlsx
@@ -2757,11 +2757,11 @@
         </is>
       </c>
       <c r="N20" s="23" t="n">
-        <v>80</v>
+        <v>95</v>
       </c>
       <c r="O20" s="24" t="inlineStr">
         <is>
-          <t>21/10: Gold 2016–2025 nạp lại trên máy N1/N2, 120 tháng, 0 lỗi: 832.436 dòng (233 s) trước khi lọc Meteostat, sau đó 788.861 dòng (292 s). 22/10: nạp lại toàn bộ 2016–2025 (176 s, 0 lỗi, DW không đổi): cả 120 file Gold lưu station_key dạng số nguyên. Bộ đặc trưng ML nằm ở gold/ml_features (ID 23); chưa có bảng pivot đa nguồn 23/10: Gold mỗi tháng gồm cả ERA5 (3 nguồn: Open-Meteo, Meteostat, ERA5). Chưa có bảng pivot đa nguồn cho ML.</t>
+          <t>21/10: Gold 2016–2025 nạp lại trên máy N1/N2, 120 tháng, 0 lỗi: 832.436 dòng (233 s) trước khi lọc Meteostat, sau đó 788.861 dòng (292 s). 22/10: nạp lại toàn bộ 2016–2025 (176 s, 0 lỗi, DW không đổi): cả 120 file Gold lưu station_key dạng số nguyên. Bộ đặc trưng ML nằm ở gold/ml_features (ID 23); chưa có bảng pivot đa nguồn 23/10: Gold mỗi tháng gồm cả ERA5 (3 nguồn: Open-Meteo, Meteostat, ERA5). Chưa có bảng pivot đa nguồn cho ML. 23/10: bảng Gold ML gộp nguồn (scripts/build_ml_pivot.py, gold/ml_pivot/weather_hourly_by_source_v1): mỗi dòng là một điểm × một giờ UTC, mỗi nguồn có cột riêng cho 8 biến (24 cột), không cộng gộp giữa các nguồn, thiếu thì để trống. 2016–2025: 701.376 dòng; số dòng, số giá trị và tổng từng cột khớp Gold, số dòng từng nguồn × năm khớp DW. Có manifest ghi nguồn gốc (SHA-256 các file Gold). Mô hình CART v1 không dùng bảng này; DW không đổi. Chờ bạn xác nhận Hoàn thành</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: clean-machine rerun evidence and reproduction guide (ID 34)
docs/reproduce-from-scratch.md lists the commands that rebuilt the
project from an empty data lake and DW on 2026-10-23, the expected
results, and the expected differences (retrieval times, Open-Meteo
generationtime_ms, surrogate keys, floating-point view sums).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Phan_cong_cong_viec_DW_khi_tuong.xlsx
+++ b/Phan_cong_cong_viec_DW_khi_tuong.xlsx
@@ -3685,13 +3685,19 @@
         <f aca="false">'Tổng quan'!$E$11+(C38-1)*7+4</f>
         <v>46367</v>
       </c>
-      <c r="M38" s="22" t="s">
-        <v>62</v>
+      <c r="M38" s="22" t="inlineStr">
+        <is>
+          <t>Đang làm</t>
+        </is>
       </c>
       <c r="N38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O38" s="24"/>
+        <v>95</v>
+      </c>
+      <c r="O38" s="24" t="inlineStr">
+        <is>
+          <t>23/10: chạy lại toàn bộ trên môi trường sạch (clone repo mới, volume Docker trống, tải lại mọi nguồn): DAG Bronze→DW 14/14 bước ngay lần đầu, 15 phút; kiểm tra chất lượng 1.032 lượt 0 lỗi; đối chiếu 1.490.237 dòng giờ, 17.866 ngày mưa. So với máy hiện tại: mọi bảng DW khớp theo khóa tự nhiên; Silver/Gold khớp từng byte; chỉ khác dấu thời gian tải và ID tự tăng. Huấn luyện lại ra đúng mô hình v1 (cùng SHA-256). Chạy lại và chạy lỗi đều đúng. Tìm ra và đã sửa 1 lỗi: trên máy mới, lệnh huấn luyện mặc định có thể lưu mô hình khác dưới tên v1; giờ v1 được ghim SHA-256 và có gói phát hành (scripts/model_release.py). Hướng dẫn: docs/reproduce-from-scratch.md. Chờ bạn xác nhận Hoàn thành</t>
+        </is>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="19" t="n">

</xml_diff>

<commit_message>
chore(workbook): mark tasks with met outputs as complete, keeping their notes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Phan_cong_cong_viec_DW_khi_tuong.xlsx
+++ b/Phan_cong_cong_viec_DW_khi_tuong.xlsx
@@ -1967,15 +1967,15 @@
       </c>
       <c r="M5" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N5" s="23" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O5" s="24" t="inlineStr">
         <is>
-          <t>22/10: kiểm chứng đầu-cuối: webserver + scheduler healthy (/health), 2 DAG nạp không lỗi, DAG kiểm tra hệ thống chạy thành công qua REST API (cả 2 task); DW giữ nguyên sau khi khởi động lại. Kiểm chứng trên 1 máy (cả nhóm hiện là 1 người). Đủ tiêu chí, chờ bạn xác nhận Hoàn thành</t>
+          <t>22/10: kiểm chứng đầu-cuối: webserver + scheduler healthy (/health), 2 DAG nạp không lỗi, DAG kiểm tra hệ thống chạy thành công qua REST API (cả 2 task); DW giữ nguyên sau khi khởi động lại. Kiểm chứng trên 1 máy (cả nhóm hiện là 1 người). Đủ tiêu chí. 23/10: dựng lại từ đầu trên môi trường sạch thành công (task 34). Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -2019,15 +2019,15 @@
       </c>
       <c r="M6" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N6" s="23" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O6" s="24" t="inlineStr">
         <is>
-          <t>22/10: 3 bucket, key đúng quy ước. Bronze Open-Meteo giữ nguyên bytes gốc + manifest (SHA-256, độ phủ, tọa độ lưới) cho cả 80 file; bỏ qua theo checksum, không theo kích thước. Còn lại: Bronze Meteostat chưa có manifest (thuộc ID 9)</t>
+          <t>22/10: 3 bucket, key đúng quy ước. Bronze Open-Meteo giữ nguyên bytes gốc + manifest (SHA-256, độ phủ, tọa độ lưới) cho cả 80 file; bỏ qua theo checksum, không theo kích thước. Còn lại: Bronze Meteostat chưa có manifest (thuộc ID 9). 23/10: Bronze Meteostat đã có manifest (task 9), phần còn lại đã xong. Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -2073,15 +2073,15 @@
       </c>
       <c r="M7" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N7" s="23" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O7" s="24" t="inlineStr">
         <is>
-          <t>22/10: sơ đồ Star Schema sinh từ DW thật (9 bảng, 14 khóa ngoại, grain từng fact): docs/diagrams/star-schema.md; thay bản phác 13/10 chỉ có trong outputs/. Cơ sở lịch UTC+7, prediction, chọn trạm (tối đa 1 trạm/điểm) đều đã chốt. Chờ bạn xác nhận Hoàn thành</t>
+          <t>22/10: sơ đồ Star Schema sinh từ DW thật (9 bảng, 14 khóa ngoại, grain từng fact): docs/diagrams/star-schema.md; thay bản phác 13/10 chỉ có trong outputs/. Cơ sở lịch UTC+7, prediction, chọn trạm (tối đa 1 trạm/điểm) đều đã chốt. Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -2127,15 +2127,15 @@
       </c>
       <c r="M8" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N8" s="23" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="O8" s="24" t="inlineStr">
         <is>
-          <t>22/10: scripts/ingest_boundaries.py: GeoJSON 63 tỉnh trước sáp nhập (geoBoundaries VNM ADM1, commit 9469f09, năm 2008) trong Bronze kèm manifest (SHA-256, giấy phép, CRS); Silver 25 tỉnh miền Bắc (QĐ 368, 369/QĐ-TTg), 8 tỉnh có dữ liệu. Hình học hợp lệ 64/64; 8/8 điểm nằm đúng tỉnh trong dim_location. Hạn chế: ranh giới lấy từ Wikipedia/Wikimedia, độ chi tiết thấp; giấy phép ghi Public Domain (geoBoundaries) và ODbL (HDX). Phạm vi đã chốt 21/10: không làm ranh giới sau sáp nhập</t>
+          <t>22/10: scripts/ingest_boundaries.py: GeoJSON 63 tỉnh trước sáp nhập (geoBoundaries VNM ADM1, commit 9469f09, năm 2008) trong Bronze kèm manifest (SHA-256, giấy phép, CRS); Silver 25 tỉnh miền Bắc (QĐ 368, 369/QĐ-TTg), 8 tỉnh có dữ liệu. Hình học hợp lệ 64/64; 8/8 điểm nằm đúng tỉnh trong dim_location. Hạn chế: ranh giới lấy từ Wikipedia/Wikimedia, độ chi tiết thấp; giấy phép ghi Public Domain (geoBoundaries) và ODbL (HDX). Phạm vi đã chốt 21/10: không làm ranh giới sau sáp nhập. Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -2179,15 +2179,15 @@
       </c>
       <c r="M9" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N9" s="23" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O9" s="24" t="inlineStr">
         <is>
-          <t>23/10: đã đăng ký CDS, chấp nhận giấy phép ERA5; yêu cầu theo vùng miền Bắc chạy được (job 70c1b649…), nhưng mỗi tháng chờ hàng đợi ~2 giờ và CDS chỉ nhận 1 yêu cầu chờ mỗi lúc. Đã chốt 23/10: dùng ERA5 time-series (cùng dữ liệu ERA5 theo giờ, ô lưới gần nhất của 8 điểm): 8 yêu cầu 2016–2025 xong trong 320 giây. Tải theo vùng vẫn chạy tiếp cho 2024–2025 để làm minh chứng. Chờ bạn xác nhận Hoàn thành</t>
+          <t>23/10: đã đăng ký CDS, chấp nhận giấy phép ERA5; yêu cầu theo vùng miền Bắc chạy được (job 70c1b649…), nhưng mỗi tháng chờ hàng đợi ~2 giờ và CDS chỉ nhận 1 yêu cầu chờ mỗi lúc. Đã chốt 23/10: dùng ERA5 time-series (cùng dữ liệu ERA5 theo giờ, ô lưới gần nhất của 8 điểm): 8 yêu cầu 2016–2025 xong trong 320 giây. Tải theo vùng vẫn chạy tiếp cho 2024–2025 để làm minh chứng. 23/10: đã dừng tải theo vùng; giữ 4 tháng (2016-01, 2016-02, 2024-01, 2024-02) làm minh chứng, dữ liệu dùng bản time-series. Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -2335,15 +2335,15 @@
       </c>
       <c r="M12" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N12" s="23" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O12" s="24" t="inlineStr">
         <is>
-          <t>22/10: Bronze giữ nguyên payload gốc + manifest; tải lại 80/80 file (339 s, 0 lỗi), dữ liệu theo giờ giống hệt bản cũ; Silver 2024 giống từng dòng (70.272). Chạy lại: bỏ qua 80 file theo checksum. Lỗi thoát mã 1 (sửa 22/10). Tiêu chí «SHA bằng bản tải mới» không đạt được về nguyên tắc vì phản hồi có generationtime_ms; thay bằng so sánh dữ liệu theo giờ</t>
+          <t>22/10: Bronze giữ nguyên payload gốc + manifest; tải lại 80/80 file (339 s, 0 lỗi), dữ liệu theo giờ giống hệt bản cũ; Silver 2024 giống từng dòng (70.272). Chạy lại: bỏ qua 80 file theo checksum. Lỗi thoát mã 1 (sửa 22/10). Tiêu chí «SHA bằng bản tải mới» không đạt được về nguyên tắc vì phản hồi có generationtime_ms; thay bằng so sánh dữ liệu theo giờ. Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -2439,15 +2439,15 @@
       </c>
       <c r="M14" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N14" s="23" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O14" s="24" t="inlineStr">
         <is>
-          <t>21/10: Silver chạy lại: Open-Meteo 701.376 dòng; Meteostat 87.485 dòng sau khi loại 436.502 giá trị mô hình và 43.575 dòng không có quan trắc; 60 file Silver cũ đã xóa; 0 xung đột, 0 lỗi. 22/10: file Bronze Open-Meteo bị thiếu tính là lỗi (trừ khi có --allow-missing); Silver kiểm tra SHA-256 của Bronze theo manifest; chạy lại Silver 2024 giống từng dòng (70.272) 23/10: Silver Open-Meteo lưu thêm tọa độ và độ cao ô lưới API trả về (grid_latitude, grid_longitude, grid_elevation_m) và báo lỗi nếu dữ liệu không ở UTC (utc_offset_seconds khác 0). Chạy lại 2016–2025: 80 file đều ở UTC, 701.376 dòng, các cột cũ giống hệt; quality gate 1.032 kiểm tra 0 lỗi; nạp lại Gold, đối chiếu 1.490.237 = 1.490.237; DW không đổi. Chờ bạn xác nhận Hoàn thành</t>
+          <t>21/10: Silver chạy lại: Open-Meteo 701.376 dòng; Meteostat 87.485 dòng sau khi loại 436.502 giá trị mô hình và 43.575 dòng không có quan trắc; 60 file Silver cũ đã xóa; 0 xung đột, 0 lỗi. 22/10: file Bronze Open-Meteo bị thiếu tính là lỗi (trừ khi có --allow-missing); Silver kiểm tra SHA-256 của Bronze theo manifest; chạy lại Silver 2024 giống từng dòng (70.272) 23/10: Silver Open-Meteo lưu thêm tọa độ và độ cao ô lưới API trả về (grid_latitude, grid_longitude, grid_elevation_m) và báo lỗi nếu dữ liệu không ở UTC (utc_offset_seconds khác 0). Chạy lại 2016–2025: 80 file đều ở UTC, 701.376 dòng, các cột cũ giống hệt; quality gate 1.032 kiểm tra 0 lỗi; nạp lại Gold, đối chiếu 1.490.237 = 1.490.237; DW không đổi. Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -2493,15 +2493,15 @@
       </c>
       <c r="M15" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N15" s="23" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O15" s="24" t="inlineStr">
         <is>
-          <t>21/10: mã/tọa độ trạm đã xác minh (Meteostat + NOAA ISD). Hợp lệ: HAN 48820, HPH 48826, TNG 48831, LCA 48803; dim_station 12 trạm (thêm 48823 Nam Định cho mưa ngày). 22/10: 48820 = sân bay Nội Bài (22,0 km, vai trò nearest_available); thêm station_role, distance_km (sql/05). Khoảng cách tính bằng haversine, không dùng GeoPandas. Tỉnh: chỉ dùng tỉnh trước sáp nhập (đã chốt 21/10); 8 điểm đã kiểm tra nằm đúng tỉnh trên GeoJSON ID 4 (22/10) 23/10: gán trạm bằng GeoPandas (scripts/assign_stations_geo.py): tính khoảng cách trên hệ tọa độ UTM 48N, trạm gần nhất trong 30 km, kiểm tra tỉnh của điểm và trạm, so với bảng trạm và dim_station (chỉ đọc). Kết quả đạt: trạm mưa GHCNh = trạm gần nhất ở cả 8 điểm; Meteostat HAN dùng Nội Bài (21,9 km) dù Hà Đông gần hơn (11,4 km, chưa chốt cho Meteostat); khoảng cách lưu lệch tối đa 0,14 km do tính trên hình cầu; 8/8 điểm đúng tỉnh. Tọa độ trạm Nội Bài nằm trong Vĩnh Phúc 2,5 km theo bản đồ geoBoundaries (chưa xác minh, không ảnh hưởng dữ liệu). DW không đổi. Chờ bạn xác nhận Hoàn thành</t>
+          <t>21/10: mã/tọa độ trạm đã xác minh (Meteostat + NOAA ISD). Hợp lệ: HAN 48820, HPH 48826, TNG 48831, LCA 48803; dim_station 12 trạm (thêm 48823 Nam Định cho mưa ngày). 22/10: 48820 = sân bay Nội Bài (22,0 km, vai trò nearest_available); thêm station_role, distance_km (sql/05). Khoảng cách tính bằng haversine, không dùng GeoPandas. Tỉnh: chỉ dùng tỉnh trước sáp nhập (đã chốt 21/10); 8 điểm đã kiểm tra nằm đúng tỉnh trên GeoJSON ID 4 (22/10) 23/10: gán trạm bằng GeoPandas (scripts/assign_stations_geo.py): tính khoảng cách trên hệ tọa độ UTM 48N, trạm gần nhất trong 30 km, kiểm tra tỉnh của điểm và trạm, so với bảng trạm và dim_station (chỉ đọc). Kết quả đạt: trạm mưa GHCNh = trạm gần nhất ở cả 8 điểm; Meteostat HAN dùng Nội Bài (21,9 km) dù Hà Đông gần hơn (11,4 km, chưa chốt cho Meteostat); khoảng cách lưu lệch tối đa 0,14 km do tính trên hình cầu; 8/8 điểm đúng tỉnh. Tọa độ trạm Nội Bài nằm trong Vĩnh Phúc 2,5 km theo bản đồ geoBoundaries (chưa xác minh, không ảnh hưởng dữ liệu). DW không đổi. Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -2545,15 +2545,15 @@
       </c>
       <c r="M16" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N16" s="23" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="O16" s="24" t="inlineStr">
         <is>
-          <t>dim_date 4.018 ngày, seed chạy lại ổn. Cơ sở lịch UTC+7 đã chốt 21/10 (data-contract, warehouse-schema; nhóm xác nhận qua N1/N2)</t>
+          <t>dim_date 4.018 ngày, seed chạy lại ổn. Cơ sở lịch UTC+7 đã chốt 21/10 (data-contract, warehouse-schema; nhóm xác nhận qua N1/N2). Hạn chế còn lại: dim_source ghi tần suất cập nhật của ERA5 là "Monthly Bulk" (thực tế tải time-series một lần); chưa sửa để giữ nguyên dữ liệu DW đã gửi Power BI. Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -2597,15 +2597,15 @@
       </c>
       <c r="M17" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N17" s="23" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="O17" s="24" t="inlineStr">
         <is>
-          <t>DDL chạy được trên Postgres; migration cho DB đã tồn tại: sql/02–05, chạy lại an toàn. 22/10: test tích hợp chạy đúng thứ tự khởi tạo thật (init + 02→05); sửa chú thích day_of_week (ISO) và period_of_day</t>
+          <t>DDL chạy được trên Postgres; migration cho DB đã tồn tại: sql/02–05, chạy lại an toàn. 22/10: test tích hợp chạy đúng thứ tự khởi tạo thật (init + 02→05); sửa chú thích day_of_week (ISO) và period_of_day. 23/10: DDL và migration 02–05 dựng DW mới thành công trên môi trường sạch (task 34). Hạn chế: tên database cố định weather_dwh. Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -2649,15 +2649,15 @@
       </c>
       <c r="M18" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N18" s="23" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O18" s="24" t="inlineStr">
         <is>
-          <t>23/10: Bronze có ERA5 NetCDF nguyên bản kèm manifest: chuỗi theo giờ 8 điểm × 2016–2025 (87.672 giờ mỗi điểm, ô lưới gần nhất; scripts/ingest_era5_timeseries.py), đọc và kiểm tra bằng xarray; khớp với file theo vùng tháng 1–2/2024 tại cùng ô lưới. Theo vùng: 2016-01, 2016-02, 2024-01, 2024-02, đang tải tiếp 2024–2025. Chạy lại: bỏ qua theo checksum. Chờ bạn xác nhận Hoàn thành</t>
+          <t>23/10: Bronze có ERA5 NetCDF nguyên bản kèm manifest: chuỗi theo giờ 8 điểm × 2016–2025 (87.672 giờ mỗi điểm, ô lưới gần nhất; scripts/ingest_era5_timeseries.py), đọc và kiểm tra bằng xarray; khớp với file theo vùng tháng 1–2/2024 tại cùng ô lưới. Theo vùng: 2016-01, 2016-02, 2024-01, 2024-02, đang tải tiếp 2024–2025. Chạy lại: bỏ qua theo checksum. 23/10: đã dừng tải theo vùng, giữ 4 tháng làm minh chứng. Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -2701,15 +2701,15 @@
       </c>
       <c r="M19" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N19" s="23" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O19" s="24" t="inlineStr">
         <is>
-          <t>23/10: scripts/transform_era5_to_silver.py: K → °C, Pa → hPa, m → mm, gió từ u/v (tốc độ và hướng gió thổi đến), mây 0–1 → %, độ ẩm tính từ nhiệt độ và điểm sương (công thức Magnus); ô lưới gần nhất ghi ở grid_latitude/grid_longitude. Mưa ERA5 theo giờ đã là tổng từng giờ nên không cần khử cộng dồn (chỉ ERA5-Land cần). 701.376 dòng, 0 giá trị bị loại. So sánh với Open-Meteo (scripts/compare_era5_open_meteo.py): nhiệt độ tương quan 0,96–0,98; áp suất ở LCA, HBI lệch nhiều do độ cao ô lưới. Chưa nạp ERA5 vào DW (chưa quyết định). Chờ bạn xác nhận Hoàn thành</t>
+          <t>23/10: scripts/transform_era5_to_silver.py: K → °C, Pa → hPa, m → mm, gió từ u/v (tốc độ và hướng gió thổi đến), mây 0–1 → %, độ ẩm tính từ nhiệt độ và điểm sương (công thức Magnus); ô lưới gần nhất ghi ở grid_latitude/grid_longitude. Mưa ERA5 theo giờ đã là tổng từng giờ nên không cần khử cộng dồn (chỉ ERA5-Land cần). 701.376 dòng, 0 giá trị bị loại. So sánh với Open-Meteo (scripts/compare_era5_open_meteo.py): nhiệt độ tương quan 0,96–0,98; áp suất ở LCA, HBI lệch nhiều do độ cao ô lưới. Chưa nạp ERA5 vào DW (chưa quyết định). 23/10: đã chốt nạp ERA5 vào DW (701.376 dòng, task 18). Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -2753,15 +2753,15 @@
       </c>
       <c r="M20" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N20" s="23" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O20" s="24" t="inlineStr">
         <is>
-          <t>21/10: Gold 2016–2025 nạp lại trên máy N1/N2, 120 tháng, 0 lỗi: 832.436 dòng (233 s) trước khi lọc Meteostat, sau đó 788.861 dòng (292 s). 22/10: nạp lại toàn bộ 2016–2025 (176 s, 0 lỗi, DW không đổi): cả 120 file Gold lưu station_key dạng số nguyên. Bộ đặc trưng ML nằm ở gold/ml_features (ID 23); chưa có bảng pivot đa nguồn 23/10: Gold mỗi tháng gồm cả ERA5 (3 nguồn: Open-Meteo, Meteostat, ERA5). Chưa có bảng pivot đa nguồn cho ML. 23/10: bảng Gold ML gộp nguồn (scripts/build_ml_pivot.py, gold/ml_pivot/weather_hourly_by_source_v1): mỗi dòng là một điểm × một giờ UTC, mỗi nguồn có cột riêng cho 8 biến (24 cột), không cộng gộp giữa các nguồn, thiếu thì để trống. 2016–2025: 701.376 dòng; số dòng, số giá trị và tổng từng cột khớp Gold, số dòng từng nguồn × năm khớp DW. Có manifest ghi nguồn gốc (SHA-256 các file Gold). Mô hình CART v1 không dùng bảng này; DW không đổi. Chờ bạn xác nhận Hoàn thành</t>
+          <t>21/10: Gold 2016–2025 nạp lại trên máy N1/N2, 120 tháng, 0 lỗi: 832.436 dòng (233 s) trước khi lọc Meteostat, sau đó 788.861 dòng (292 s). 22/10: nạp lại toàn bộ 2016–2025 (176 s, 0 lỗi, DW không đổi): cả 120 file Gold lưu station_key dạng số nguyên. Bộ đặc trưng ML nằm ở gold/ml_features (ID 23); chưa có bảng pivot đa nguồn 23/10: Gold mỗi tháng gồm cả ERA5 (3 nguồn: Open-Meteo, Meteostat, ERA5). Chưa có bảng pivot đa nguồn cho ML. 23/10: bảng Gold ML gộp nguồn (scripts/build_ml_pivot.py, gold/ml_pivot/weather_hourly_by_source_v1): mỗi dòng là một điểm × một giờ UTC, mỗi nguồn có cột riêng cho 8 biến (24 cột), không cộng gộp giữa các nguồn, thiếu thì để trống. 2016–2025: 701.376 dòng; số dòng, số giá trị và tổng từng cột khớp Gold, số dòng từng nguồn × năm khớp DW. Có manifest ghi nguồn gốc (SHA-256 các file Gold). Mô hình CART v1 không dùng bảng này; DW không đổi. Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -2807,15 +2807,15 @@
       </c>
       <c r="M21" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N21" s="23" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O21" s="24" t="inlineStr">
         <is>
-          <t>22/10: dags/dag_weather_pipeline.py (weather_bronze_to_dw_dag): Open-Meteo, Meteostat, mưa ngày GHCNh: tải → Silver → seed dim → Gold/DW → đối chiếu DW với Silver (scripts/reconcile_dw.py). Tham số năm 2016–2025 và điểm; chạy tay, 1 lượt một lúc. Đã chạy: 2024 HAN, chạy lại không thêm dòng, cố ý tắt MinIO rồi chạy tiếp thành công, 2024 cả 8 điểm, và cả 2016–2025 (3 phút 43 giây; khớp 788.861 dòng giờ và 17.866 ngày mưa; không tải lại gì). Cửa sổ nhỏ nhất 1 năm × 1 điểm (đã chốt). Chờ bạn xác nhận Hoàn thành 23/10: thêm nhánh ERA5 (tải time-series → Silver) trước bước quality_gate. Chạy 2016–2025: 14/14 task thành công (lần đầu bước ERA5 lỗi vì container Airflow chưa có khóa CDS; đã sửa, chạy tiếp từ bước lỗi); đối chiếu 1.490.237 = 1.490.237 dòng giờ, 17.866 = 17.866 ngày mưa.</t>
+          <t>22/10: dags/dag_weather_pipeline.py (weather_bronze_to_dw_dag): Open-Meteo, Meteostat, mưa ngày GHCNh: tải → Silver → seed dim → Gold/DW → đối chiếu DW với Silver (scripts/reconcile_dw.py). Tham số năm 2016–2025 và điểm; chạy tay, 1 lượt một lúc. Đã chạy: 2024 HAN, chạy lại không thêm dòng, cố ý tắt MinIO rồi chạy tiếp thành công, 2024 cả 8 điểm, và cả 2016–2025 (3 phút 43 giây; khớp 788.861 dòng giờ và 17.866 ngày mưa; không tải lại gì). Cửa sổ nhỏ nhất 1 năm × 1 điểm (đã chốt). 23/10: thêm nhánh ERA5 (tải time-series → Silver) trước bước quality_gate. Chạy 2016–2025: 14/14 task thành công (lần đầu bước ERA5 lỗi vì container Airflow chưa có khóa CDS; đã sửa, chạy tiếp từ bước lỗi); đối chiếu 1.490.237 = 1.490.237 dòng giờ, 17.866 = 17.866 ngày mưa. Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -2859,15 +2859,15 @@
       </c>
       <c r="M22" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N22" s="23" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O22" s="24" t="inlineStr">
         <is>
-          <t>21/10: DW sạch: 788.861 dòng (Open-Meteo 701.376 + Meteostat HAN 87.485), 0 trùng khóa; rút dòng sai đã kiểm chứng trên dữ liệu thật; lần nạp cuối 292 s (bản trước ghi 3.493 s là sai). 22/10: phạm vi xóa khi nạp lại tính theo phạm vi yêu cầu (nguồn biến mất bị xóa; thiếu file Silver Open-Meteo của một vị trí thì tháng đó báo lỗi); thêm pressure_type (sql/05). Chạy lại 2024 trên trạng thái hiện tại: 79.039 dòng, không đổi. Bản 994.145 dòng trên máy bacnx đã lỗi thời 23/10: nạp thêm ERA5 701.376 dòng (đã chốt nạp ERA5 theo đề cương §8, §10); DW 1.490.237 dòng, 0 trùng khóa; Open-Meteo, Meteostat, mưa ngày, dự báo không đổi.</t>
+          <t>21/10: DW sạch: 788.861 dòng (Open-Meteo 701.376 + Meteostat HAN 87.485), 0 trùng khóa; rút dòng sai đã kiểm chứng trên dữ liệu thật; lần nạp cuối 292 s (bản trước ghi 3.493 s là sai). 22/10: phạm vi xóa khi nạp lại tính theo phạm vi yêu cầu (nguồn biến mất bị xóa; thiếu file Silver Open-Meteo của một vị trí thì tháng đó báo lỗi); thêm pressure_type (sql/05). Chạy lại 2024 trên trạng thái hiện tại: 79.039 dòng, không đổi. Bản 994.145 dòng trên máy bacnx đã lỗi thời 23/10: nạp thêm ERA5 701.376 dòng (đã chốt nạp ERA5 theo đề cương §8, §10); DW 1.490.237 dòng, 0 trùng khóa; Open-Meteo, Meteostat, mưa ngày, dự báo không đổi. Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -2911,15 +2911,15 @@
       </c>
       <c r="M23" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N23" s="23" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="O23" s="24" t="inlineStr">
         <is>
-          <t>21/10: sql/02_olap_views.sql (6 view giờ/ngày/tháng/năm/độ phủ), ngày mưa ≥1 mm, ngày nóng ≥35 °C; đối soát giờ→ngày→tháng→năm khớp 0 chênh trên 788.861 dòng; 3 test tích hợp. Chưa dùng trong Power BI</t>
+          <t>21/10: sql/02_olap_views.sql (6 view giờ/ngày/tháng/năm/độ phủ), ngày mưa ≥1 mm, ngày nóng ≥35 °C; đối soát giờ→ngày→tháng→năm khớp 0 chênh trên 788.861 dòng; 3 test tích hợp. Chưa dùng trong Power BI. 23/10: view có trong gói Power BI đã gửi (DW 1.490.237 dòng); dựng lại đúng trên môi trường sạch (task 34). Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -3171,15 +3171,15 @@
       </c>
       <c r="M28" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N28" s="23" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O28" s="24" t="inlineStr">
         <is>
-          <t>22/10: scripts/quality_gate.py, task quality_gate trong DAG (sau bước Silver, trước khi ghi DW). Dừng DAG khi: thiếu cột hoặc khóa trống; giờ không UTC hoặc sai tháng; trùng nguồn × điểm × giờ; giá trị ngoài khoảng hợp lệ của data-contract; thiếu giờ Open-Meteo; GHCNh trùng ngày, sai khung 12:00 UTC, mưa ngoài 0–999 mm. Cảnh báo, không dừng (ngưỡng chốt 22/10 từ dữ liệu 2016–2025): độ phủ Meteostat &lt; 95%, GHCNh &lt; 90%; Open-Meteo thiếu giá trị; Meteostat thiếu nhiệt độ/độ ẩm &gt; 5%; nhiệt độ ngoài 0–45 °C; áp suất ngoài 950–1050 hPa; mưa giờ &gt; 100 mm; mưa ngày ≥ 300 mm chưa duyệt. Dữ liệu thật 2016–2025: 712 kiểm tra, 0 lỗi, 0 cảnh báo; DAG 2024 HAN 12/12 task; test tích hợp xác nhận task Airflow báo lỗi khi Silver sai. Chờ bạn xác nhận Hoàn thành 23/10: kiểm tra cả ERA5 (bắt buộc đủ giờ; cảnh báo áp suất ngoài 900–1050 hPa vì ô lưới cao hơn điểm): 1.032 kiểm tra, 0 lỗi, 0 cảnh báo.</t>
+          <t>22/10: scripts/quality_gate.py, task quality_gate trong DAG (sau bước Silver, trước khi ghi DW). Dừng DAG khi: thiếu cột hoặc khóa trống; giờ không UTC hoặc sai tháng; trùng nguồn × điểm × giờ; giá trị ngoài khoảng hợp lệ của data-contract; thiếu giờ Open-Meteo; GHCNh trùng ngày, sai khung 12:00 UTC, mưa ngoài 0–999 mm. Cảnh báo, không dừng (ngưỡng chốt 22/10 từ dữ liệu 2016–2025): độ phủ Meteostat &lt; 95%, GHCNh &lt; 90%; Open-Meteo thiếu giá trị; Meteostat thiếu nhiệt độ/độ ẩm &gt; 5%; nhiệt độ ngoài 0–45 °C; áp suất ngoài 950–1050 hPa; mưa giờ &gt; 100 mm; mưa ngày ≥ 300 mm chưa duyệt. Dữ liệu thật 2016–2025: 712 kiểm tra, 0 lỗi, 0 cảnh báo; DAG 2024 HAN 12/12 task; test tích hợp xác nhận task Airflow báo lỗi khi Silver sai. 23/10: kiểm tra cả ERA5 (bắt buộc đủ giờ; cảnh báo áp suất ngoài 900–1050 hPa vì ô lưới cao hơn điểm): 1.032 kiểm tra, 0 lỗi, 0 cảnh báo. Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -3223,15 +3223,15 @@
       </c>
       <c r="M29" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N29" s="23" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>23/10: DAG weather_incremental_dag chạy theo lịch hằng ngày (không chạy bù quá khứ, tạm dừng khi mới tạo): đọc mốc watermark trong MinIO (năm cuối đã nạp và đối chiếu xong) → chọn năm mới tiếp theo + chạy lại 1 năm trước để lấy dữ liệu sửa muộn, không vượt quá 2025 → gọi DAG Bronze→DW (task 17) và chờ → chỉ dời mốc khi lần chạy đó thành công. Chạy thật: đặt mốc 2024, lần chạy theo lịch xử lý 2024–2025 (14/14 task, 3 phút, đối chiếu 298.192 = 298.192 dòng giờ), mốc dời lên 2025; DW giống hệt trước khi chạy (không trùng, không đổi giá trị); lần chạy sau tự bỏ qua vì đã đủ đến 2025. Chờ bạn xác nhận Hoàn thành</t>
+          <t>23/10: DAG weather_incremental_dag chạy theo lịch hằng ngày (không chạy bù quá khứ, tạm dừng khi mới tạo): đọc mốc watermark trong MinIO (năm cuối đã nạp và đối chiếu xong) → chọn năm mới tiếp theo + chạy lại 1 năm trước để lấy dữ liệu sửa muộn, không vượt quá 2025 → gọi DAG Bronze→DW (task 17) và chờ → chỉ dời mốc khi lần chạy đó thành công. Chạy thật: đặt mốc 2024, lần chạy theo lịch xử lý 2024–2025 (14/14 task, 3 phút, đối chiếu 298.192 = 298.192 dòng giờ), mốc dời lên 2025; DW giống hệt trước khi chạy (không trùng, không đổi giá trị); lần chạy sau tự bỏ qua vì đã đủ đến 2025. Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -3277,15 +3277,15 @@
       </c>
       <c r="M30" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N30" s="23" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O30" s="24" t="inlineStr">
         <is>
-          <t>23/10: đo thật bằng scripts/benchmark_dw_queries.py (EXPLAIN ANALYZE, 3 lần, trung vị) trên DW 1.490.237 dòng: nạp từng view cho dashboard 0,3–1,3 giây, tổng khoảng 5,8 giây; truy vấn đối chiếu 0,4 ms–1,2 giây. Index hiện có đã đủ cho truy vấn có lọc; đã thử thêm index ghép và index cho 4 khóa ngoại trong giao dịch rồi hoàn tác: không nhanh hơn (view tổng hợp phải quét cả bảng), nên không thêm. Mục tiêu đã chốt 23/10: mỗi view dưới 5 giây, truy vấn đối chiếu dưới 2 giây (đang đạt: tối đa 1,3 giây và 1,2 giây). Chờ bạn xác nhận Hoàn thành</t>
+          <t>23/10: đo thật bằng scripts/benchmark_dw_queries.py (EXPLAIN ANALYZE, 3 lần, trung vị) trên DW 1.490.237 dòng: nạp từng view cho dashboard 0,3–1,3 giây, tổng khoảng 5,8 giây; truy vấn đối chiếu 0,4 ms–1,2 giây. Index hiện có đã đủ cho truy vấn có lọc; đã thử thêm index ghép và index cho 4 khóa ngoại trong giao dịch rồi hoàn tác: không nhanh hơn (view tổng hợp phải quét cả bảng), nên không thêm. Mục tiêu đã chốt 23/10: mỗi view dưới 5 giây, truy vấn đối chiếu dưới 2 giây (đang đạt: tối đa 1,3 giây và 1,2 giây). Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -3533,15 +3533,15 @@
       </c>
       <c r="M35" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N35" s="23" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>22/10: sql/04_predictions.sql (dim_model, khóa duy nhất model × vị trí × origin UTC, cửa sổ mục tiêu, view vw_prediction_vs_actual) + scripts/load_predictions.py. Đã nạp 69.888 dự đoán test 2025, chạy lại không trùng. View đối chiếu đã phát hiện lỗi nhãn ID 22 (đã sửa); ma trận nhầm lẫn DW = kết quả chấm lại. sql/05: dim_model ghi rõ nhãn của từng chỉ số (chọn trên v0.2, F1 val 0,786; test trên v0.2.1, F1 val trên nhãn này 0,789). Do N1/N2 làm thay N3</t>
+          <t>22/10: sql/04_predictions.sql (dim_model, khóa duy nhất model × vị trí × origin UTC, cửa sổ mục tiêu, view vw_prediction_vs_actual) + scripts/load_predictions.py. Đã nạp 69.888 dự đoán test 2025, chạy lại không trùng. View đối chiếu đã phát hiện lỗi nhãn ID 22 (đã sửa); ma trận nhầm lẫn DW = kết quả chấm lại. sql/05: dim_model ghi rõ nhãn của từng chỉ số (chọn trên v0.2, F1 val 0,786; test trên v0.2.1, F1 val trên nhãn này 0,789). Do N1/N2 làm thay N3. 23/10: dựng lại đúng trên môi trường sạch (task 34). Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -3587,15 +3587,15 @@
       </c>
       <c r="M36" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N36" s="23" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O36" s="24" t="inlineStr">
         <is>
-          <t>23/10: DAG weather_rain_scoring_dag (chạy tay): kiểm tra khoảng ngày → chấm điểm (scripts/score_cart.py: kiểm tra SHA-256 của mô hình, tính lại đặc trưng từ Silver, thiếu dữ liệu thì báo lỗi) → ghi Gold mỗi ngày một file → đăng lên DW (scripts/publish_predictions.py: chỉ ghi dòng thay đổi) → đối chiếu DW với Gold. Chỉ đăng dự báo tập test 2025 (01/01–30/12, mục tiêu không sang 2026). Chạy thật cả năm 2025: 4/4 task thành công trong 40 giây, 69.888 dự báo, DW không đổi dòng nào (mã băm trước và sau giống hệt); thử khoảng ngày sai thì DAG dừng ngay ở bước đầu. Chờ bạn xác nhận Hoàn thành</t>
+          <t>23/10: DAG weather_rain_scoring_dag (chạy tay): kiểm tra khoảng ngày → chấm điểm (scripts/score_cart.py: kiểm tra SHA-256 của mô hình, tính lại đặc trưng từ Silver, thiếu dữ liệu thì báo lỗi) → ghi Gold mỗi ngày một file → đăng lên DW (scripts/publish_predictions.py: chỉ ghi dòng thay đổi) → đối chiếu DW với Gold. Chỉ đăng dự báo tập test 2025 (01/01–30/12, mục tiêu không sang 2026). Chạy thật cả năm 2025: 4/4 task thành công trong 40 giây, 69.888 dự báo, DW không đổi dòng nào (mã băm trước và sau giống hệt); thử khoảng ngày sai thì DAG dừng ngay ở bước đầu. Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -3687,15 +3687,15 @@
       </c>
       <c r="M38" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N38" s="23" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O38" s="24" t="inlineStr">
         <is>
-          <t>23/10: chạy lại toàn bộ trên môi trường sạch (clone repo mới, volume Docker trống, tải lại mọi nguồn): DAG Bronze→DW 14/14 bước ngay lần đầu, 15 phút; kiểm tra chất lượng 1.032 lượt 0 lỗi; đối chiếu 1.490.237 dòng giờ, 17.866 ngày mưa. So với máy hiện tại: mọi bảng DW khớp theo khóa tự nhiên; Silver/Gold khớp từng byte; chỉ khác dấu thời gian tải và ID tự tăng. Huấn luyện lại ra đúng mô hình v1 (cùng SHA-256). Chạy lại và chạy lỗi đều đúng. Tìm ra và đã sửa 1 lỗi: trên máy mới, lệnh huấn luyện mặc định có thể lưu mô hình khác dưới tên v1; giờ v1 được ghim SHA-256 và có gói phát hành (scripts/model_release.py). Hướng dẫn: docs/reproduce-from-scratch.md. Chờ bạn xác nhận Hoàn thành</t>
+          <t>23/10: chạy lại toàn bộ trên môi trường sạch (clone repo mới, volume Docker trống, tải lại mọi nguồn): DAG Bronze→DW 14/14 bước ngay lần đầu, 15 phút; kiểm tra chất lượng 1.032 lượt 0 lỗi; đối chiếu 1.490.237 dòng giờ, 17.866 ngày mưa. So với máy hiện tại: mọi bảng DW khớp theo khóa tự nhiên; Silver/Gold khớp từng byte; chỉ khác dấu thời gian tải và ID tự tăng. Huấn luyện lại ra đúng mô hình v1 (cùng SHA-256). Chạy lại và chạy lỗi đều đúng. Tìm ra và đã sửa 1 lỗi: trên máy mới, lệnh huấn luyện mặc định có thể lưu mô hình khác dưới tên v1; giờ v1 được ghim SHA-256 và có gói phát hành (scripts/model_release.py). Hướng dẫn: docs/reproduce-from-scratch.md. Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: record the N3 review of the ML decisions and the 300 mm rule
All eight ML checklist items and the GHCNh unsupported-extreme rule were
confirmed on 2026-10-23; the workbook marks IDs 9, 21-23, 28-30 and 36
complete with their notes kept.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Phan_cong_cong_viec_DW_khi_tuong.xlsx
+++ b/Phan_cong_cong_viec_DW_khi_tuong.xlsx
@@ -2291,7 +2291,7 @@
       </c>
       <c r="O11" s="24" t="inlineStr">
         <is>
-          <t>Hoàn thành 21/10: rain-label.md v0.2: ngưỡng 1 mm, nguồn Open-Meteo, cửa sổ (t,t+24h] đã kiểm chứng, thiếu giờ thì bỏ nhãn. Tỷ lệ Yes 50,5% đo bằng bản v0.2; bản v0.2.1 (sửa lỗi cộng số thực 22/10): train 51,6% / val 50,1% / test 49,7%. Nhóm xác nhận qua N1/N2; N3 chưa duyệt. Còn mở có ghi rõ: fallback ERA5/trạm, ngưỡng độ phủ tối thiểu</t>
+          <t>Hoàn thành 21/10: rain-label.md v0.2: ngưỡng 1 mm, nguồn Open-Meteo, cửa sổ (t,t+24h] đã kiểm chứng, thiếu giờ thì bỏ nhãn. Tỷ lệ Yes 50,5% đo bằng bản v0.2; bản v0.2.1 (sửa lỗi cộng số thực 22/10): train 51,6% / val 50,1% / test 49,7%. Nhóm xác nhận qua N1/N2; N3 chưa duyệt. Còn mở có ghi rõ: fallback ERA5/trạm, ngưỡng độ phủ tối thiểu. 23/10: N3 đã duyệt.</t>
         </is>
       </c>
     </row>
@@ -2387,15 +2387,15 @@
       </c>
       <c r="M13" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N13" s="23" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O13" s="24" t="inlineStr">
         <is>
-          <t>21/10: Meteostat chỉ giữ quan trắc thật (HAN). NOAA GHCNh mưa 24h cho 5 điểm (HPH, TNG, LCA, HAN≈Hà Đông, NBI≈Nam Định) 2016–2025: 17.866 ngày, độ phủ 95,9–99,2%, bảng fact_station_daily_rain + view so sánh với Open-Meteo. 22/10: trạm Meteostat 48820 thực chất là sân bay Nội Bài (cách điểm HAN 22 km), đã ghi lại; quy tắc cực trị so sánh theo độ phân giải 0,1 mm. Bronze Meteostat lưu CSV đã giải nén, chưa có manifest/SHA. Chờ nhóm duyệt quy tắc cực trị 300 mm 23/10: Bronze Meteostat lưu nguyên file .csv.gz nhận về kèm manifest (SHA-256, URL, thời điểm tải); 15 file CSV cũ được thay sau khi kiểm tra bản tải mới giải nén giống hệt từng byte; 25 năm-trạm không có dữ liệu (HTTP 404) được ghi lại nên lần sau không hỏi lại. Silver Meteostat kiểm tra SHA-256, chạy lại giống hệt (120 file, 87.485 dòng); DW không đổi. Chạy chuỗi DAG 2024 × HAN trong container không có Internet: 13/13 bước thành công.</t>
+          <t>21/10: Meteostat chỉ giữ quan trắc thật (HAN). NOAA GHCNh mưa 24h cho 5 điểm (HPH, TNG, LCA, HAN≈Hà Đông, NBI≈Nam Định) 2016–2025: 17.866 ngày, độ phủ 95,9–99,2%, bảng fact_station_daily_rain + view so sánh với Open-Meteo. 22/10: trạm Meteostat 48820 thực chất là sân bay Nội Bài (cách điểm HAN 22 km), đã ghi lại; quy tắc cực trị so sánh theo độ phân giải 0,1 mm. Bronze Meteostat lưu CSV đã giải nén, chưa có manifest/SHA. Quy tắc cực trị 300 mm chờ nhóm duyệt. 23/10: Bronze Meteostat lưu nguyên file .csv.gz nhận về kèm manifest (SHA-256, URL, thời điểm tải); 15 file CSV cũ được thay sau khi kiểm tra bản tải mới giải nén giống hệt từng byte; 25 năm-trạm không có dữ liệu (HTTP 404) được ghi lại nên lần sau không hỏi lại. Silver Meteostat kiểm tra SHA-256, chạy lại giống hệt (120 file, 87.485 dòng); DW không đổi. Chạy chuỗi DAG 2024 × HAN trong container không có Internet: 13/13 bước thành công. 23/10: đã duyệt quy tắc cực trị 300 mm (2016–2025 chỉ cách ly 1 ngày: Nam Định 13/10/2023, 700 mm; giữ 2 trận có thật 491,3 mm và 338 mm). Ngưỡng 300 mm và 10% là ngưỡng nhóm tự đặt. Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -3015,15 +3015,15 @@
       </c>
       <c r="M25" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N25" s="23" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>22/10: notebooks/eda_rain_next24h.ipynb (nhãn đã sửa), chỉ dùng train để chọn biến: mùa vụ mạnh theo tháng giờ Việt Nam (T8 78,6%, T12 26,5%; bản trước dùng tháng UTC), giờ trong ngày gần như không ảnh hưởng (51,3-52,0%), biến tách tốt nhất: điểm sương, mưa 24h trước, độ ẩm. Thêm bảng tương quan Spearman: cặp mạnh độ ẩm–chênh điểm sương (-1,00), nhiệt độ–điểm sương (0,87), điểm sương–áp suất (-0,80). Logic trong scripts/rain_eda.py có test. Do N1/N2 làm thay N3</t>
+          <t>22/10: notebooks/eda_rain_next24h.ipynb (nhãn đã sửa), chỉ dùng train để chọn biến: mùa vụ mạnh theo tháng giờ Việt Nam (T8 78,6%, T12 26,5%; bản trước dùng tháng UTC), giờ trong ngày gần như không ảnh hưởng (51,3-52,0%), biến tách tốt nhất: điểm sương, mưa 24h trước, độ ẩm. Thêm bảng tương quan Spearman: cặp mạnh độ ẩm–chênh điểm sương (-1,00), nhiệt độ–điểm sương (0,87), điểm sương–áp suất (-0,80). Logic trong scripts/rain_eda.py có test. Do N1/N2 làm thay N3. 23/10: N3 đã duyệt 8 mục quyết định ML trong rain-label.md. Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -3067,15 +3067,15 @@
       </c>
       <c r="M26" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N26" s="23" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O26" s="24" t="inlineStr">
         <is>
-          <t>22/10: nhãn v2 (rain_next24h_v0.2.1) gold/ml_labels/rain_next24h_labels_v2.parquet: 700.800 nhãn dùng được, Yes 51,6% / 50,1% / 49,7% (train/val/test), 576 loại ở ranh giới. Đã sửa lỗi cộng số thực: bản v1 gán Không mưa cho 5.147 cửa sổ đúng 1,0 mm (0,73%); phát hiện nhờ đối chiếu DW ở ID 31. Có test hồi quy. Do N1/N2 làm thay N3</t>
+          <t>22/10: nhãn v2 (rain_next24h_v0.2.1) gold/ml_labels/rain_next24h_labels_v2.parquet: 700.800 nhãn dùng được, Yes 51,6% / 50,1% / 49,7% (train/val/test), 576 loại ở ranh giới. Đã sửa lỗi cộng số thực: bản v1 gán Không mưa cho 5.147 cửa sổ đúng 1,0 mm (0,73%); phát hiện nhờ đối chiếu DW ở ID 31. Có test hồi quy. Do N1/N2 làm thay N3. 23/10: N3 đã duyệt 8 mục quyết định ML trong rain-label.md. Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -3119,15 +3119,15 @@
       </c>
       <c r="M27" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N27" s="23" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>22/10: đặc trưng v2 gold/ml_features/cart_rain_{train_2016_2023,val_2024,test_2025}_v2.parquet + manifest (nhãn v0.2.1, tổng mưa làm tròn); v1 giữ cho model v1. 22 đặc trưng chỉ từ Open-Meteo, 700.800 dòng; thiếu chỉ ở 24 giờ đầu 2016. Test chống rò rỉ, thiếu giờ, không lẫn vị trí. Do N1/N2 làm thay N3</t>
+          <t>22/10: đặc trưng v2 gold/ml_features/cart_rain_{train_2016_2023,val_2024,test_2025}_v2.parquet + manifest (nhãn v0.2.1, tổng mưa làm tròn); v1 giữ cho model v1. 22 đặc trưng chỉ từ Open-Meteo, 700.800 dòng; thiếu chỉ ở 24 giờ đầu 2016. Test chống rò rỉ, thiếu giờ, không lẫn vị trí. Do N1/N2 làm thay N3. 23/10: N3 đã duyệt 8 mục quyết định ML trong rain-label.md. Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -3375,15 +3375,15 @@
       </c>
       <c r="M32" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N32" s="23" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="O32" s="24" t="inlineStr">
         <is>
-          <t>21/10: gold/ml_models/cart_rain_next24h_v1 (model.joblib + report.json). Lưới 120 cấu hình, chọn trên validation 2024: max_depth=8, min_samples_leaf=50, class_weight=balanced, ccp_alpha=1e-4, 88 lá, ngưỡng 0,40. Validation (nhãn đã sửa 22/10): Precision 0,760 / Recall 0,819 / F1 0,789. Model train trên nhãn v1 (0,73% sai), không train lại để giữ test độc lập. 22/10: chặn ghi đè model (model đã chấm test thì không cho ghi đè). Chọn cấu hình và ngưỡng theo F1. Quy tắc ưu tiên Recall đã chốt 22/10: ngưỡng 0,36 (Recall validation 0,88); 0,40 vẫn là kết quả test chính thức. Chờ N3 duyệt (rain-label.md). Do N1/N2 làm thay N3</t>
+          <t>21/10: gold/ml_models/cart_rain_next24h_v1 (model.joblib + report.json). Lưới 120 cấu hình, chọn trên validation 2024: max_depth=8, min_samples_leaf=50, class_weight=balanced, ccp_alpha=1e-4, 88 lá, ngưỡng 0,40. Validation (nhãn đã sửa 22/10): Precision 0,760 / Recall 0,819 / F1 0,789. Model train trên nhãn v1 (0,73% sai), không train lại để giữ test độc lập. 22/10: chặn ghi đè model (model đã chấm test thì không cho ghi đè). Chọn cấu hình và ngưỡng theo F1. Quy tắc ưu tiên Recall đã chốt 22/10: ngưỡng 0,36 (Recall validation 0,88); 0,40 vẫn là kết quả test chính thức. Do N1/N2 làm thay N3. 23/10: N3 đã duyệt 8 mục quyết định ML trong rain-label.md. Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -3427,15 +3427,15 @@
       </c>
       <c r="M33" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N33" s="23" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>22/10: đánh giá 1 lần trên test 2025, model + ngưỡng 0,40 chốt từ validation. Chấm lại với nhãn đã sửa (dự đoán giữ nguyên, kiểm SHA-256 model): TP 27.467 / FP 8.569 / TN 26.617 / FN 7.235; Accuracy 0,774, Precision 0,762, Recall 0,792, F1 0,777 (dự báo theo hiện trạng F1 0,729). Mùa mưa F1 0,836, mùa khô 0,624. Khớp hoàn toàn với view DW. test_predictions.parquet giữ nhãn cũ v0.2: phân tích lấy nhãn từ đặc trưng v2. Do N1/N2 làm thay N3</t>
+          <t>22/10: đánh giá 1 lần trên test 2025, model + ngưỡng 0,40 chốt từ validation. Chấm lại với nhãn đã sửa (dự đoán giữ nguyên, kiểm SHA-256 model): TP 27.467 / FP 8.569 / TN 26.617 / FN 7.235; Accuracy 0,774, Precision 0,762, Recall 0,792, F1 0,777 (dự báo theo hiện trạng F1 0,729). Mùa mưa F1 0,836, mùa khô 0,624. Khớp hoàn toàn với view DW. test_predictions.parquet giữ nhãn cũ v0.2: phân tích lấy nhãn từ đặc trưng v2. Do N1/N2 làm thay N3. 23/10: N3 đã duyệt 8 mục quyết định ML trong rain-label.md. Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -3479,15 +3479,15 @@
       </c>
       <c r="M34" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N34" s="23" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="O34" s="24" t="inlineStr">
         <is>
-          <t>22/10: notebooks/cart_tree_rules.ipynb (SHA-256 đúng model ID 29): hình 3 tầng đầu, 88 luật bằng tên + đơn vị thật, độ quan trọng, 4 ví dụ test 2025, hồ sơ ca bỏ sót trên validation (nhãn đã sửa): 65% dưới 5 mm, 55% xác suất 0,30-0,40, mưa sau 24h khô chỉ bắt được 17% (mùa khô 2,5%). Đã sửa lời diễn giải «mưa không báo trước». Ý tưởng thêm hướng gió đến từ một ví dụ test 2025: phải chứng minh bằng EDA trên train trước. Do N1/N2 làm thay N3</t>
+          <t>22/10: notebooks/cart_tree_rules.ipynb (SHA-256 đúng model ID 29): hình 3 tầng đầu, 88 luật bằng tên + đơn vị thật, độ quan trọng, 4 ví dụ test 2025, hồ sơ ca bỏ sót trên validation (nhãn đã sửa): 65% dưới 5 mm, 55% xác suất 0,30-0,40, mưa sau 24h khô chỉ bắt được 17% (mùa khô 2,5%). Đã sửa lời diễn giải «mưa không báo trước». Ý tưởng thêm hướng gió đến từ một ví dụ test 2025: phải chứng minh bằng EDA trên train trước. Do N1/N2 làm thay N3. 23/10: N3 đã duyệt 8 mục quyết định ML trong rain-label.md. Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>
@@ -3785,15 +3785,15 @@
       </c>
       <c r="M40" s="22" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="N40" s="23" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O40" s="24" t="inlineStr">
         <is>
-          <t>23/10: scripts/analyze_cart_thresholds.py → gold/ml_models/cart_rain_next24h_v1/threshold_error_analysis.json. So sánh ngưỡng trên validation 2024 (lưới 0,30–0,70 của quy tắc chọn ngưỡng): quy tắc F1 vẫn ra 0,40 (ngưỡng chính thức), quy tắc ưu tiên Recall ra 0,36. Test 2025 chỉ tính ở các ngưỡng đã chốt (phân tích sau, có ghi rõ): 0,40 → P 0,762 / R 0,792 / F1 0,777; 0,36 → 0,723 / 0,848 / 0,780 (thêm 2.709 báo động giả, bớt 1.945 ca bỏ sót). Lỗi: bỏ sót nhiều nhất ở mưa nhẹ 1–2 mm (42%); báo động giả phần lớn là cửa sổ có 0–1 mm; mưa sau 24 giờ khô chỉ bắt được 17%; mùa mưa F1 0,836, mùa khô 0,624. Chi tiết: rain-label.md. Do N1/N2 làm thay N3. Chờ bạn xác nhận Hoàn thành</t>
+          <t>23/10: scripts/analyze_cart_thresholds.py → gold/ml_models/cart_rain_next24h_v1/threshold_error_analysis.json. So sánh ngưỡng trên validation 2024 (lưới 0,30–0,70 của quy tắc chọn ngưỡng): quy tắc F1 vẫn ra 0,40 (ngưỡng chính thức), quy tắc ưu tiên Recall ra 0,36. Test 2025 chỉ tính ở các ngưỡng đã chốt (phân tích sau, có ghi rõ): 0,40 → P 0,762 / R 0,792 / F1 0,777; 0,36 → 0,723 / 0,848 / 0,780 (thêm 2.709 báo động giả, bớt 1.945 ca bỏ sót). Lỗi: bỏ sót nhiều nhất ở mưa nhẹ 1–2 mm (42%); báo động giả phần lớn là cửa sổ có 0–1 mm; mưa sau 24 giờ khô chỉ bắt được 17%; mùa mưa F1 0,836, mùa khô 0,624. Chi tiết: rain-label.md. Do N1/N2 làm thay N3. 23/10: N3 đã duyệt 8 mục quyết định ML trong rain-label.md. Xác nhận Hoàn thành 23/10.</t>
         </is>
       </c>
     </row>

</xml_diff>